<commit_message>
fix: alinear HTML y Excel de la calculadora Temporal Cloud tras revisión de pares
Usa GB decimal (KB/1e6), origen vacío como Cliente, y evita que localStorage en file:// tumbe el recálculo.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/temporal-cloud-calculator/calculadora-temporal-cloud.xlsx
+++ b/temporal-cloud-calculator/calculadora-temporal-cloud.xlsx
@@ -711,7 +711,7 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>6. Storage activo = exec × (KB/1024/1024) × horas open. Retenido = exec × GB × días × 24. Régimen mensual, no invoice.</t>
+          <t>6. Storage: 1 GB = 1.000.000 KB. Activo = exec × (KB/1e6) × horas open. Retenido = exec × GB × días × 24. Nombres de workflow unicos (SUMIF).</t>
         </is>
       </c>
     </row>
@@ -916,13 +916,30 @@
           <t>TOTAL USD / mes</t>
         </is>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C12" s="14">
         <f>N(C6)+N(C9)+N(C10)</f>
         <v/>
       </c>
-      <c r="C12" s="14">
-        <f>B12</f>
-        <v/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Nombres duplicados en Workflows (0 = OK)</t>
+        </is>
+      </c>
+      <c r="B13" s="7">
+        <f>SUMPRODUCT((Workflows!A2:A21&lt;&gt;"")*(COUNTIF(Workflows!A2:A21,Workflows!A2:A21)&gt;1))</f>
+        <v/>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1245,7 +1262,7 @@
         </is>
       </c>
       <c r="D2" s="7">
-        <f>IF(A2="","",IF(C2="Cliente",1,IF(C2="Signal-With-Start",1,IF(C2="Schedule",3,0))))</f>
+        <f>IF(A2="","",IF(C2="Signal-With-Start",1,IF(C2="Schedule",3,IF(C2="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E2" s="19" t="n">
@@ -1262,15 +1279,15 @@
         <v/>
       </c>
       <c r="I2" s="9">
-        <f>IF(A2="","",B2*(D2+H2))</f>
+        <f>IF(A2="","",MAX(0,N(B2))*(D2+H2))</f>
         <v/>
       </c>
       <c r="J2" s="11">
-        <f>IF(A2="","",B2*(F2/1024/1024)*E2)</f>
+        <f>IF(A2="","",MAX(0,N(B2))*(MAX(0,N(F2))/1000000)*MAX(0,N(E2)))</f>
         <v/>
       </c>
       <c r="K2" s="11">
-        <f>IF(A2="","",B2*(F2/1024/1024)*G2*24)</f>
+        <f>IF(A2="","",MAX(0,N(B2))*(MAX(0,N(F2))/1000000)*MAX(0,N(G2))*24)</f>
         <v/>
       </c>
       <c r="L2" s="10">
@@ -1305,7 +1322,7 @@
         </is>
       </c>
       <c r="D3" s="7">
-        <f>IF(A3="","",IF(C3="Cliente",1,IF(C3="Signal-With-Start",1,IF(C3="Schedule",3,0))))</f>
+        <f>IF(A3="","",IF(C3="Signal-With-Start",1,IF(C3="Schedule",3,IF(C3="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E3" s="19" t="n">
@@ -1322,15 +1339,15 @@
         <v/>
       </c>
       <c r="I3" s="9">
-        <f>IF(A3="","",B3*(D3+H3))</f>
+        <f>IF(A3="","",MAX(0,N(B3))*(D3+H3))</f>
         <v/>
       </c>
       <c r="J3" s="11">
-        <f>IF(A3="","",B3*(F3/1024/1024)*E3)</f>
+        <f>IF(A3="","",MAX(0,N(B3))*(MAX(0,N(F3))/1000000)*MAX(0,N(E3)))</f>
         <v/>
       </c>
       <c r="K3" s="11">
-        <f>IF(A3="","",B3*(F3/1024/1024)*G3*24)</f>
+        <f>IF(A3="","",MAX(0,N(B3))*(MAX(0,N(F3))/1000000)*MAX(0,N(G3))*24)</f>
         <v/>
       </c>
       <c r="L3" s="10">
@@ -1355,7 +1372,7 @@
       <c r="B4" s="18" t="n"/>
       <c r="C4" s="17" t="inlineStr"/>
       <c r="D4" s="7">
-        <f>IF(A4="","",IF(C4="Cliente",1,IF(C4="Signal-With-Start",1,IF(C4="Schedule",3,0))))</f>
+        <f>IF(A4="","",IF(C4="Signal-With-Start",1,IF(C4="Schedule",3,IF(C4="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E4" s="19" t="n"/>
@@ -1366,15 +1383,15 @@
         <v/>
       </c>
       <c r="I4" s="9">
-        <f>IF(A4="","",B4*(D4+H4))</f>
+        <f>IF(A4="","",MAX(0,N(B4))*(D4+H4))</f>
         <v/>
       </c>
       <c r="J4" s="11">
-        <f>IF(A4="","",B4*(F4/1024/1024)*E4)</f>
+        <f>IF(A4="","",MAX(0,N(B4))*(MAX(0,N(F4))/1000000)*MAX(0,N(E4)))</f>
         <v/>
       </c>
       <c r="K4" s="11">
-        <f>IF(A4="","",B4*(F4/1024/1024)*G4*24)</f>
+        <f>IF(A4="","",MAX(0,N(B4))*(MAX(0,N(F4))/1000000)*MAX(0,N(G4))*24)</f>
         <v/>
       </c>
       <c r="L4" s="10">
@@ -1399,7 +1416,7 @@
       <c r="B5" s="18" t="n"/>
       <c r="C5" s="17" t="inlineStr"/>
       <c r="D5" s="7">
-        <f>IF(A5="","",IF(C5="Cliente",1,IF(C5="Signal-With-Start",1,IF(C5="Schedule",3,0))))</f>
+        <f>IF(A5="","",IF(C5="Signal-With-Start",1,IF(C5="Schedule",3,IF(C5="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E5" s="19" t="n"/>
@@ -1410,15 +1427,15 @@
         <v/>
       </c>
       <c r="I5" s="9">
-        <f>IF(A5="","",B5*(D5+H5))</f>
+        <f>IF(A5="","",MAX(0,N(B5))*(D5+H5))</f>
         <v/>
       </c>
       <c r="J5" s="11">
-        <f>IF(A5="","",B5*(F5/1024/1024)*E5)</f>
+        <f>IF(A5="","",MAX(0,N(B5))*(MAX(0,N(F5))/1000000)*MAX(0,N(E5)))</f>
         <v/>
       </c>
       <c r="K5" s="11">
-        <f>IF(A5="","",B5*(F5/1024/1024)*G5*24)</f>
+        <f>IF(A5="","",MAX(0,N(B5))*(MAX(0,N(F5))/1000000)*MAX(0,N(G5))*24)</f>
         <v/>
       </c>
       <c r="L5" s="10">
@@ -1443,7 +1460,7 @@
       <c r="B6" s="18" t="n"/>
       <c r="C6" s="17" t="inlineStr"/>
       <c r="D6" s="7">
-        <f>IF(A6="","",IF(C6="Cliente",1,IF(C6="Signal-With-Start",1,IF(C6="Schedule",3,0))))</f>
+        <f>IF(A6="","",IF(C6="Signal-With-Start",1,IF(C6="Schedule",3,IF(C6="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E6" s="19" t="n"/>
@@ -1454,15 +1471,15 @@
         <v/>
       </c>
       <c r="I6" s="9">
-        <f>IF(A6="","",B6*(D6+H6))</f>
+        <f>IF(A6="","",MAX(0,N(B6))*(D6+H6))</f>
         <v/>
       </c>
       <c r="J6" s="11">
-        <f>IF(A6="","",B6*(F6/1024/1024)*E6)</f>
+        <f>IF(A6="","",MAX(0,N(B6))*(MAX(0,N(F6))/1000000)*MAX(0,N(E6)))</f>
         <v/>
       </c>
       <c r="K6" s="11">
-        <f>IF(A6="","",B6*(F6/1024/1024)*G6*24)</f>
+        <f>IF(A6="","",MAX(0,N(B6))*(MAX(0,N(F6))/1000000)*MAX(0,N(G6))*24)</f>
         <v/>
       </c>
       <c r="L6" s="10">
@@ -1487,7 +1504,7 @@
       <c r="B7" s="18" t="n"/>
       <c r="C7" s="17" t="inlineStr"/>
       <c r="D7" s="7">
-        <f>IF(A7="","",IF(C7="Cliente",1,IF(C7="Signal-With-Start",1,IF(C7="Schedule",3,0))))</f>
+        <f>IF(A7="","",IF(C7="Signal-With-Start",1,IF(C7="Schedule",3,IF(C7="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E7" s="19" t="n"/>
@@ -1498,15 +1515,15 @@
         <v/>
       </c>
       <c r="I7" s="9">
-        <f>IF(A7="","",B7*(D7+H7))</f>
+        <f>IF(A7="","",MAX(0,N(B7))*(D7+H7))</f>
         <v/>
       </c>
       <c r="J7" s="11">
-        <f>IF(A7="","",B7*(F7/1024/1024)*E7)</f>
+        <f>IF(A7="","",MAX(0,N(B7))*(MAX(0,N(F7))/1000000)*MAX(0,N(E7)))</f>
         <v/>
       </c>
       <c r="K7" s="11">
-        <f>IF(A7="","",B7*(F7/1024/1024)*G7*24)</f>
+        <f>IF(A7="","",MAX(0,N(B7))*(MAX(0,N(F7))/1000000)*MAX(0,N(G7))*24)</f>
         <v/>
       </c>
       <c r="L7" s="10">
@@ -1531,7 +1548,7 @@
       <c r="B8" s="18" t="n"/>
       <c r="C8" s="17" t="inlineStr"/>
       <c r="D8" s="7">
-        <f>IF(A8="","",IF(C8="Cliente",1,IF(C8="Signal-With-Start",1,IF(C8="Schedule",3,0))))</f>
+        <f>IF(A8="","",IF(C8="Signal-With-Start",1,IF(C8="Schedule",3,IF(C8="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E8" s="19" t="n"/>
@@ -1542,15 +1559,15 @@
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>IF(A8="","",B8*(D8+H8))</f>
+        <f>IF(A8="","",MAX(0,N(B8))*(D8+H8))</f>
         <v/>
       </c>
       <c r="J8" s="11">
-        <f>IF(A8="","",B8*(F8/1024/1024)*E8)</f>
+        <f>IF(A8="","",MAX(0,N(B8))*(MAX(0,N(F8))/1000000)*MAX(0,N(E8)))</f>
         <v/>
       </c>
       <c r="K8" s="11">
-        <f>IF(A8="","",B8*(F8/1024/1024)*G8*24)</f>
+        <f>IF(A8="","",MAX(0,N(B8))*(MAX(0,N(F8))/1000000)*MAX(0,N(G8))*24)</f>
         <v/>
       </c>
       <c r="L8" s="10">
@@ -1575,7 +1592,7 @@
       <c r="B9" s="18" t="n"/>
       <c r="C9" s="17" t="inlineStr"/>
       <c r="D9" s="7">
-        <f>IF(A9="","",IF(C9="Cliente",1,IF(C9="Signal-With-Start",1,IF(C9="Schedule",3,0))))</f>
+        <f>IF(A9="","",IF(C9="Signal-With-Start",1,IF(C9="Schedule",3,IF(C9="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E9" s="19" t="n"/>
@@ -1586,15 +1603,15 @@
         <v/>
       </c>
       <c r="I9" s="9">
-        <f>IF(A9="","",B9*(D9+H9))</f>
+        <f>IF(A9="","",MAX(0,N(B9))*(D9+H9))</f>
         <v/>
       </c>
       <c r="J9" s="11">
-        <f>IF(A9="","",B9*(F9/1024/1024)*E9)</f>
+        <f>IF(A9="","",MAX(0,N(B9))*(MAX(0,N(F9))/1000000)*MAX(0,N(E9)))</f>
         <v/>
       </c>
       <c r="K9" s="11">
-        <f>IF(A9="","",B9*(F9/1024/1024)*G9*24)</f>
+        <f>IF(A9="","",MAX(0,N(B9))*(MAX(0,N(F9))/1000000)*MAX(0,N(G9))*24)</f>
         <v/>
       </c>
       <c r="L9" s="10">
@@ -1619,7 +1636,7 @@
       <c r="B10" s="18" t="n"/>
       <c r="C10" s="17" t="inlineStr"/>
       <c r="D10" s="7">
-        <f>IF(A10="","",IF(C10="Cliente",1,IF(C10="Signal-With-Start",1,IF(C10="Schedule",3,0))))</f>
+        <f>IF(A10="","",IF(C10="Signal-With-Start",1,IF(C10="Schedule",3,IF(C10="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E10" s="19" t="n"/>
@@ -1630,15 +1647,15 @@
         <v/>
       </c>
       <c r="I10" s="9">
-        <f>IF(A10="","",B10*(D10+H10))</f>
+        <f>IF(A10="","",MAX(0,N(B10))*(D10+H10))</f>
         <v/>
       </c>
       <c r="J10" s="11">
-        <f>IF(A10="","",B10*(F10/1024/1024)*E10)</f>
+        <f>IF(A10="","",MAX(0,N(B10))*(MAX(0,N(F10))/1000000)*MAX(0,N(E10)))</f>
         <v/>
       </c>
       <c r="K10" s="11">
-        <f>IF(A10="","",B10*(F10/1024/1024)*G10*24)</f>
+        <f>IF(A10="","",MAX(0,N(B10))*(MAX(0,N(F10))/1000000)*MAX(0,N(G10))*24)</f>
         <v/>
       </c>
       <c r="L10" s="10">
@@ -1663,7 +1680,7 @@
       <c r="B11" s="18" t="n"/>
       <c r="C11" s="17" t="inlineStr"/>
       <c r="D11" s="7">
-        <f>IF(A11="","",IF(C11="Cliente",1,IF(C11="Signal-With-Start",1,IF(C11="Schedule",3,0))))</f>
+        <f>IF(A11="","",IF(C11="Signal-With-Start",1,IF(C11="Schedule",3,IF(C11="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E11" s="19" t="n"/>
@@ -1674,15 +1691,15 @@
         <v/>
       </c>
       <c r="I11" s="9">
-        <f>IF(A11="","",B11*(D11+H11))</f>
+        <f>IF(A11="","",MAX(0,N(B11))*(D11+H11))</f>
         <v/>
       </c>
       <c r="J11" s="11">
-        <f>IF(A11="","",B11*(F11/1024/1024)*E11)</f>
+        <f>IF(A11="","",MAX(0,N(B11))*(MAX(0,N(F11))/1000000)*MAX(0,N(E11)))</f>
         <v/>
       </c>
       <c r="K11" s="11">
-        <f>IF(A11="","",B11*(F11/1024/1024)*G11*24)</f>
+        <f>IF(A11="","",MAX(0,N(B11))*(MAX(0,N(F11))/1000000)*MAX(0,N(G11))*24)</f>
         <v/>
       </c>
       <c r="L11" s="10">
@@ -1707,7 +1724,7 @@
       <c r="B12" s="18" t="n"/>
       <c r="C12" s="17" t="inlineStr"/>
       <c r="D12" s="7">
-        <f>IF(A12="","",IF(C12="Cliente",1,IF(C12="Signal-With-Start",1,IF(C12="Schedule",3,0))))</f>
+        <f>IF(A12="","",IF(C12="Signal-With-Start",1,IF(C12="Schedule",3,IF(C12="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E12" s="19" t="n"/>
@@ -1718,15 +1735,15 @@
         <v/>
       </c>
       <c r="I12" s="9">
-        <f>IF(A12="","",B12*(D12+H12))</f>
+        <f>IF(A12="","",MAX(0,N(B12))*(D12+H12))</f>
         <v/>
       </c>
       <c r="J12" s="11">
-        <f>IF(A12="","",B12*(F12/1024/1024)*E12)</f>
+        <f>IF(A12="","",MAX(0,N(B12))*(MAX(0,N(F12))/1000000)*MAX(0,N(E12)))</f>
         <v/>
       </c>
       <c r="K12" s="11">
-        <f>IF(A12="","",B12*(F12/1024/1024)*G12*24)</f>
+        <f>IF(A12="","",MAX(0,N(B12))*(MAX(0,N(F12))/1000000)*MAX(0,N(G12))*24)</f>
         <v/>
       </c>
       <c r="L12" s="10">
@@ -1751,7 +1768,7 @@
       <c r="B13" s="18" t="n"/>
       <c r="C13" s="17" t="inlineStr"/>
       <c r="D13" s="7">
-        <f>IF(A13="","",IF(C13="Cliente",1,IF(C13="Signal-With-Start",1,IF(C13="Schedule",3,0))))</f>
+        <f>IF(A13="","",IF(C13="Signal-With-Start",1,IF(C13="Schedule",3,IF(C13="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E13" s="19" t="n"/>
@@ -1762,15 +1779,15 @@
         <v/>
       </c>
       <c r="I13" s="9">
-        <f>IF(A13="","",B13*(D13+H13))</f>
+        <f>IF(A13="","",MAX(0,N(B13))*(D13+H13))</f>
         <v/>
       </c>
       <c r="J13" s="11">
-        <f>IF(A13="","",B13*(F13/1024/1024)*E13)</f>
+        <f>IF(A13="","",MAX(0,N(B13))*(MAX(0,N(F13))/1000000)*MAX(0,N(E13)))</f>
         <v/>
       </c>
       <c r="K13" s="11">
-        <f>IF(A13="","",B13*(F13/1024/1024)*G13*24)</f>
+        <f>IF(A13="","",MAX(0,N(B13))*(MAX(0,N(F13))/1000000)*MAX(0,N(G13))*24)</f>
         <v/>
       </c>
       <c r="L13" s="10">
@@ -1795,7 +1812,7 @@
       <c r="B14" s="18" t="n"/>
       <c r="C14" s="17" t="inlineStr"/>
       <c r="D14" s="7">
-        <f>IF(A14="","",IF(C14="Cliente",1,IF(C14="Signal-With-Start",1,IF(C14="Schedule",3,0))))</f>
+        <f>IF(A14="","",IF(C14="Signal-With-Start",1,IF(C14="Schedule",3,IF(C14="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E14" s="19" t="n"/>
@@ -1806,15 +1823,15 @@
         <v/>
       </c>
       <c r="I14" s="9">
-        <f>IF(A14="","",B14*(D14+H14))</f>
+        <f>IF(A14="","",MAX(0,N(B14))*(D14+H14))</f>
         <v/>
       </c>
       <c r="J14" s="11">
-        <f>IF(A14="","",B14*(F14/1024/1024)*E14)</f>
+        <f>IF(A14="","",MAX(0,N(B14))*(MAX(0,N(F14))/1000000)*MAX(0,N(E14)))</f>
         <v/>
       </c>
       <c r="K14" s="11">
-        <f>IF(A14="","",B14*(F14/1024/1024)*G14*24)</f>
+        <f>IF(A14="","",MAX(0,N(B14))*(MAX(0,N(F14))/1000000)*MAX(0,N(G14))*24)</f>
         <v/>
       </c>
       <c r="L14" s="10">
@@ -1839,7 +1856,7 @@
       <c r="B15" s="18" t="n"/>
       <c r="C15" s="17" t="inlineStr"/>
       <c r="D15" s="7">
-        <f>IF(A15="","",IF(C15="Cliente",1,IF(C15="Signal-With-Start",1,IF(C15="Schedule",3,0))))</f>
+        <f>IF(A15="","",IF(C15="Signal-With-Start",1,IF(C15="Schedule",3,IF(C15="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E15" s="19" t="n"/>
@@ -1850,15 +1867,15 @@
         <v/>
       </c>
       <c r="I15" s="9">
-        <f>IF(A15="","",B15*(D15+H15))</f>
+        <f>IF(A15="","",MAX(0,N(B15))*(D15+H15))</f>
         <v/>
       </c>
       <c r="J15" s="11">
-        <f>IF(A15="","",B15*(F15/1024/1024)*E15)</f>
+        <f>IF(A15="","",MAX(0,N(B15))*(MAX(0,N(F15))/1000000)*MAX(0,N(E15)))</f>
         <v/>
       </c>
       <c r="K15" s="11">
-        <f>IF(A15="","",B15*(F15/1024/1024)*G15*24)</f>
+        <f>IF(A15="","",MAX(0,N(B15))*(MAX(0,N(F15))/1000000)*MAX(0,N(G15))*24)</f>
         <v/>
       </c>
       <c r="L15" s="10">
@@ -1883,7 +1900,7 @@
       <c r="B16" s="18" t="n"/>
       <c r="C16" s="17" t="inlineStr"/>
       <c r="D16" s="7">
-        <f>IF(A16="","",IF(C16="Cliente",1,IF(C16="Signal-With-Start",1,IF(C16="Schedule",3,0))))</f>
+        <f>IF(A16="","",IF(C16="Signal-With-Start",1,IF(C16="Schedule",3,IF(C16="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E16" s="19" t="n"/>
@@ -1894,15 +1911,15 @@
         <v/>
       </c>
       <c r="I16" s="9">
-        <f>IF(A16="","",B16*(D16+H16))</f>
+        <f>IF(A16="","",MAX(0,N(B16))*(D16+H16))</f>
         <v/>
       </c>
       <c r="J16" s="11">
-        <f>IF(A16="","",B16*(F16/1024/1024)*E16)</f>
+        <f>IF(A16="","",MAX(0,N(B16))*(MAX(0,N(F16))/1000000)*MAX(0,N(E16)))</f>
         <v/>
       </c>
       <c r="K16" s="11">
-        <f>IF(A16="","",B16*(F16/1024/1024)*G16*24)</f>
+        <f>IF(A16="","",MAX(0,N(B16))*(MAX(0,N(F16))/1000000)*MAX(0,N(G16))*24)</f>
         <v/>
       </c>
       <c r="L16" s="10">
@@ -1927,7 +1944,7 @@
       <c r="B17" s="18" t="n"/>
       <c r="C17" s="17" t="inlineStr"/>
       <c r="D17" s="7">
-        <f>IF(A17="","",IF(C17="Cliente",1,IF(C17="Signal-With-Start",1,IF(C17="Schedule",3,0))))</f>
+        <f>IF(A17="","",IF(C17="Signal-With-Start",1,IF(C17="Schedule",3,IF(C17="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E17" s="19" t="n"/>
@@ -1938,15 +1955,15 @@
         <v/>
       </c>
       <c r="I17" s="9">
-        <f>IF(A17="","",B17*(D17+H17))</f>
+        <f>IF(A17="","",MAX(0,N(B17))*(D17+H17))</f>
         <v/>
       </c>
       <c r="J17" s="11">
-        <f>IF(A17="","",B17*(F17/1024/1024)*E17)</f>
+        <f>IF(A17="","",MAX(0,N(B17))*(MAX(0,N(F17))/1000000)*MAX(0,N(E17)))</f>
         <v/>
       </c>
       <c r="K17" s="11">
-        <f>IF(A17="","",B17*(F17/1024/1024)*G17*24)</f>
+        <f>IF(A17="","",MAX(0,N(B17))*(MAX(0,N(F17))/1000000)*MAX(0,N(G17))*24)</f>
         <v/>
       </c>
       <c r="L17" s="10">
@@ -1971,7 +1988,7 @@
       <c r="B18" s="18" t="n"/>
       <c r="C18" s="17" t="inlineStr"/>
       <c r="D18" s="7">
-        <f>IF(A18="","",IF(C18="Cliente",1,IF(C18="Signal-With-Start",1,IF(C18="Schedule",3,0))))</f>
+        <f>IF(A18="","",IF(C18="Signal-With-Start",1,IF(C18="Schedule",3,IF(C18="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E18" s="19" t="n"/>
@@ -1982,15 +1999,15 @@
         <v/>
       </c>
       <c r="I18" s="9">
-        <f>IF(A18="","",B18*(D18+H18))</f>
+        <f>IF(A18="","",MAX(0,N(B18))*(D18+H18))</f>
         <v/>
       </c>
       <c r="J18" s="11">
-        <f>IF(A18="","",B18*(F18/1024/1024)*E18)</f>
+        <f>IF(A18="","",MAX(0,N(B18))*(MAX(0,N(F18))/1000000)*MAX(0,N(E18)))</f>
         <v/>
       </c>
       <c r="K18" s="11">
-        <f>IF(A18="","",B18*(F18/1024/1024)*G18*24)</f>
+        <f>IF(A18="","",MAX(0,N(B18))*(MAX(0,N(F18))/1000000)*MAX(0,N(G18))*24)</f>
         <v/>
       </c>
       <c r="L18" s="10">
@@ -2015,7 +2032,7 @@
       <c r="B19" s="18" t="n"/>
       <c r="C19" s="17" t="inlineStr"/>
       <c r="D19" s="7">
-        <f>IF(A19="","",IF(C19="Cliente",1,IF(C19="Signal-With-Start",1,IF(C19="Schedule",3,0))))</f>
+        <f>IF(A19="","",IF(C19="Signal-With-Start",1,IF(C19="Schedule",3,IF(C19="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E19" s="19" t="n"/>
@@ -2026,15 +2043,15 @@
         <v/>
       </c>
       <c r="I19" s="9">
-        <f>IF(A19="","",B19*(D19+H19))</f>
+        <f>IF(A19="","",MAX(0,N(B19))*(D19+H19))</f>
         <v/>
       </c>
       <c r="J19" s="11">
-        <f>IF(A19="","",B19*(F19/1024/1024)*E19)</f>
+        <f>IF(A19="","",MAX(0,N(B19))*(MAX(0,N(F19))/1000000)*MAX(0,N(E19)))</f>
         <v/>
       </c>
       <c r="K19" s="11">
-        <f>IF(A19="","",B19*(F19/1024/1024)*G19*24)</f>
+        <f>IF(A19="","",MAX(0,N(B19))*(MAX(0,N(F19))/1000000)*MAX(0,N(G19))*24)</f>
         <v/>
       </c>
       <c r="L19" s="10">
@@ -2059,7 +2076,7 @@
       <c r="B20" s="18" t="n"/>
       <c r="C20" s="17" t="inlineStr"/>
       <c r="D20" s="7">
-        <f>IF(A20="","",IF(C20="Cliente",1,IF(C20="Signal-With-Start",1,IF(C20="Schedule",3,0))))</f>
+        <f>IF(A20="","",IF(C20="Signal-With-Start",1,IF(C20="Schedule",3,IF(C20="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E20" s="19" t="n"/>
@@ -2070,15 +2087,15 @@
         <v/>
       </c>
       <c r="I20" s="9">
-        <f>IF(A20="","",B20*(D20+H20))</f>
+        <f>IF(A20="","",MAX(0,N(B20))*(D20+H20))</f>
         <v/>
       </c>
       <c r="J20" s="11">
-        <f>IF(A20="","",B20*(F20/1024/1024)*E20)</f>
+        <f>IF(A20="","",MAX(0,N(B20))*(MAX(0,N(F20))/1000000)*MAX(0,N(E20)))</f>
         <v/>
       </c>
       <c r="K20" s="11">
-        <f>IF(A20="","",B20*(F20/1024/1024)*G20*24)</f>
+        <f>IF(A20="","",MAX(0,N(B20))*(MAX(0,N(F20))/1000000)*MAX(0,N(G20))*24)</f>
         <v/>
       </c>
       <c r="L20" s="10">
@@ -2103,7 +2120,7 @@
       <c r="B21" s="18" t="n"/>
       <c r="C21" s="17" t="inlineStr"/>
       <c r="D21" s="7">
-        <f>IF(A21="","",IF(C21="Cliente",1,IF(C21="Signal-With-Start",1,IF(C21="Schedule",3,0))))</f>
+        <f>IF(A21="","",IF(C21="Signal-With-Start",1,IF(C21="Schedule",3,IF(C21="Ninguno",0,1))))</f>
         <v/>
       </c>
       <c r="E21" s="19" t="n"/>
@@ -2114,15 +2131,15 @@
         <v/>
       </c>
       <c r="I21" s="9">
-        <f>IF(A21="","",B21*(D21+H21))</f>
+        <f>IF(A21="","",MAX(0,N(B21))*(D21+H21))</f>
         <v/>
       </c>
       <c r="J21" s="11">
-        <f>IF(A21="","",B21*(F21/1024/1024)*E21)</f>
+        <f>IF(A21="","",MAX(0,N(B21))*(MAX(0,N(F21))/1000000)*MAX(0,N(E21)))</f>
         <v/>
       </c>
       <c r="K21" s="11">
-        <f>IF(A21="","",B21*(F21/1024/1024)*G21*24)</f>
+        <f>IF(A21="","",MAX(0,N(B21))*(MAX(0,N(F21))/1000000)*MAX(0,N(G21))*24)</f>
         <v/>
       </c>
       <c r="L21" s="10">
@@ -2254,7 +2271,7 @@
         <v/>
       </c>
       <c r="I2" s="22">
-        <f>IF(OR(A2="",B2=""),"",IF(B2="Activity",D2*(E2/100)*(1+N(F2)+N(G2)),D2*(E2/100)*H2))</f>
+        <f>IF(OR(A2="",B2=""),"",IF(B2="Activity",MAX(0,N(D2))*(MIN(100,MAX(0,N(E2)))/100)*(1+MAX(0,N(F2))+MAX(0,N(G2))),MAX(0,N(D2))*(MIN(100,MAX(0,N(E2)))/100)*H2))</f>
         <v/>
       </c>
     </row>
@@ -2291,7 +2308,7 @@
         <v/>
       </c>
       <c r="I3" s="22">
-        <f>IF(OR(A3="",B3=""),"",IF(B3="Activity",D3*(E3/100)*(1+N(F3)+N(G3)),D3*(E3/100)*H3))</f>
+        <f>IF(OR(A3="",B3=""),"",IF(B3="Activity",MAX(0,N(D3))*(MIN(100,MAX(0,N(E3)))/100)*(1+MAX(0,N(F3))+MAX(0,N(G3))),MAX(0,N(D3))*(MIN(100,MAX(0,N(E3)))/100)*H3))</f>
         <v/>
       </c>
     </row>
@@ -2328,7 +2345,7 @@
         <v/>
       </c>
       <c r="I4" s="22">
-        <f>IF(OR(A4="",B4=""),"",IF(B4="Activity",D4*(E4/100)*(1+N(F4)+N(G4)),D4*(E4/100)*H4))</f>
+        <f>IF(OR(A4="",B4=""),"",IF(B4="Activity",MAX(0,N(D4))*(MIN(100,MAX(0,N(E4)))/100)*(1+MAX(0,N(F4))+MAX(0,N(G4))),MAX(0,N(D4))*(MIN(100,MAX(0,N(E4)))/100)*H4))</f>
         <v/>
       </c>
     </row>
@@ -2365,7 +2382,7 @@
         <v/>
       </c>
       <c r="I5" s="22">
-        <f>IF(OR(A5="",B5=""),"",IF(B5="Activity",D5*(E5/100)*(1+N(F5)+N(G5)),D5*(E5/100)*H5))</f>
+        <f>IF(OR(A5="",B5=""),"",IF(B5="Activity",MAX(0,N(D5))*(MIN(100,MAX(0,N(E5)))/100)*(1+MAX(0,N(F5))+MAX(0,N(G5))),MAX(0,N(D5))*(MIN(100,MAX(0,N(E5)))/100)*H5))</f>
         <v/>
       </c>
     </row>
@@ -2402,7 +2419,7 @@
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>IF(OR(A6="",B6=""),"",IF(B6="Activity",D6*(E6/100)*(1+N(F6)+N(G6)),D6*(E6/100)*H6))</f>
+        <f>IF(OR(A6="",B6=""),"",IF(B6="Activity",MAX(0,N(D6))*(MIN(100,MAX(0,N(E6)))/100)*(1+MAX(0,N(F6))+MAX(0,N(G6))),MAX(0,N(D6))*(MIN(100,MAX(0,N(E6)))/100)*H6))</f>
         <v/>
       </c>
     </row>
@@ -2439,7 +2456,7 @@
         <v/>
       </c>
       <c r="I7" s="22">
-        <f>IF(OR(A7="",B7=""),"",IF(B7="Activity",D7*(E7/100)*(1+N(F7)+N(G7)),D7*(E7/100)*H7))</f>
+        <f>IF(OR(A7="",B7=""),"",IF(B7="Activity",MAX(0,N(D7))*(MIN(100,MAX(0,N(E7)))/100)*(1+MAX(0,N(F7))+MAX(0,N(G7))),MAX(0,N(D7))*(MIN(100,MAX(0,N(E7)))/100)*H7))</f>
         <v/>
       </c>
     </row>
@@ -2476,7 +2493,7 @@
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>IF(OR(A8="",B8=""),"",IF(B8="Activity",D8*(E8/100)*(1+N(F8)+N(G8)),D8*(E8/100)*H8))</f>
+        <f>IF(OR(A8="",B8=""),"",IF(B8="Activity",MAX(0,N(D8))*(MIN(100,MAX(0,N(E8)))/100)*(1+MAX(0,N(F8))+MAX(0,N(G8))),MAX(0,N(D8))*(MIN(100,MAX(0,N(E8)))/100)*H8))</f>
         <v/>
       </c>
     </row>
@@ -2513,7 +2530,7 @@
         <v/>
       </c>
       <c r="I9" s="22">
-        <f>IF(OR(A9="",B9=""),"",IF(B9="Activity",D9*(E9/100)*(1+N(F9)+N(G9)),D9*(E9/100)*H9))</f>
+        <f>IF(OR(A9="",B9=""),"",IF(B9="Activity",MAX(0,N(D9))*(MIN(100,MAX(0,N(E9)))/100)*(1+MAX(0,N(F9))+MAX(0,N(G9))),MAX(0,N(D9))*(MIN(100,MAX(0,N(E9)))/100)*H9))</f>
         <v/>
       </c>
     </row>
@@ -2550,7 +2567,7 @@
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>IF(OR(A10="",B10=""),"",IF(B10="Activity",D10*(E10/100)*(1+N(F10)+N(G10)),D10*(E10/100)*H10))</f>
+        <f>IF(OR(A10="",B10=""),"",IF(B10="Activity",MAX(0,N(D10))*(MIN(100,MAX(0,N(E10)))/100)*(1+MAX(0,N(F10))+MAX(0,N(G10))),MAX(0,N(D10))*(MIN(100,MAX(0,N(E10)))/100)*H10))</f>
         <v/>
       </c>
     </row>
@@ -2587,7 +2604,7 @@
         <v/>
       </c>
       <c r="I11" s="22">
-        <f>IF(OR(A11="",B11=""),"",IF(B11="Activity",D11*(E11/100)*(1+N(F11)+N(G11)),D11*(E11/100)*H11))</f>
+        <f>IF(OR(A11="",B11=""),"",IF(B11="Activity",MAX(0,N(D11))*(MIN(100,MAX(0,N(E11)))/100)*(1+MAX(0,N(F11))+MAX(0,N(G11))),MAX(0,N(D11))*(MIN(100,MAX(0,N(E11)))/100)*H11))</f>
         <v/>
       </c>
     </row>
@@ -2624,7 +2641,7 @@
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>IF(OR(A12="",B12=""),"",IF(B12="Activity",D12*(E12/100)*(1+N(F12)+N(G12)),D12*(E12/100)*H12))</f>
+        <f>IF(OR(A12="",B12=""),"",IF(B12="Activity",MAX(0,N(D12))*(MIN(100,MAX(0,N(E12)))/100)*(1+MAX(0,N(F12))+MAX(0,N(G12))),MAX(0,N(D12))*(MIN(100,MAX(0,N(E12)))/100)*H12))</f>
         <v/>
       </c>
     </row>
@@ -2661,7 +2678,7 @@
         <v/>
       </c>
       <c r="I13" s="22">
-        <f>IF(OR(A13="",B13=""),"",IF(B13="Activity",D13*(E13/100)*(1+N(F13)+N(G13)),D13*(E13/100)*H13))</f>
+        <f>IF(OR(A13="",B13=""),"",IF(B13="Activity",MAX(0,N(D13))*(MIN(100,MAX(0,N(E13)))/100)*(1+MAX(0,N(F13))+MAX(0,N(G13))),MAX(0,N(D13))*(MIN(100,MAX(0,N(E13)))/100)*H13))</f>
         <v/>
       </c>
     </row>
@@ -2678,7 +2695,7 @@
         <v/>
       </c>
       <c r="I14" s="22">
-        <f>IF(OR(A14="",B14=""),"",IF(B14="Activity",D14*(E14/100)*(1+N(F14)+N(G14)),D14*(E14/100)*H14))</f>
+        <f>IF(OR(A14="",B14=""),"",IF(B14="Activity",MAX(0,N(D14))*(MIN(100,MAX(0,N(E14)))/100)*(1+MAX(0,N(F14))+MAX(0,N(G14))),MAX(0,N(D14))*(MIN(100,MAX(0,N(E14)))/100)*H14))</f>
         <v/>
       </c>
     </row>
@@ -2695,7 +2712,7 @@
         <v/>
       </c>
       <c r="I15" s="22">
-        <f>IF(OR(A15="",B15=""),"",IF(B15="Activity",D15*(E15/100)*(1+N(F15)+N(G15)),D15*(E15/100)*H15))</f>
+        <f>IF(OR(A15="",B15=""),"",IF(B15="Activity",MAX(0,N(D15))*(MIN(100,MAX(0,N(E15)))/100)*(1+MAX(0,N(F15))+MAX(0,N(G15))),MAX(0,N(D15))*(MIN(100,MAX(0,N(E15)))/100)*H15))</f>
         <v/>
       </c>
     </row>
@@ -2712,7 +2729,7 @@
         <v/>
       </c>
       <c r="I16" s="22">
-        <f>IF(OR(A16="",B16=""),"",IF(B16="Activity",D16*(E16/100)*(1+N(F16)+N(G16)),D16*(E16/100)*H16))</f>
+        <f>IF(OR(A16="",B16=""),"",IF(B16="Activity",MAX(0,N(D16))*(MIN(100,MAX(0,N(E16)))/100)*(1+MAX(0,N(F16))+MAX(0,N(G16))),MAX(0,N(D16))*(MIN(100,MAX(0,N(E16)))/100)*H16))</f>
         <v/>
       </c>
     </row>
@@ -2729,7 +2746,7 @@
         <v/>
       </c>
       <c r="I17" s="22">
-        <f>IF(OR(A17="",B17=""),"",IF(B17="Activity",D17*(E17/100)*(1+N(F17)+N(G17)),D17*(E17/100)*H17))</f>
+        <f>IF(OR(A17="",B17=""),"",IF(B17="Activity",MAX(0,N(D17))*(MIN(100,MAX(0,N(E17)))/100)*(1+MAX(0,N(F17))+MAX(0,N(G17))),MAX(0,N(D17))*(MIN(100,MAX(0,N(E17)))/100)*H17))</f>
         <v/>
       </c>
     </row>
@@ -2746,7 +2763,7 @@
         <v/>
       </c>
       <c r="I18" s="22">
-        <f>IF(OR(A18="",B18=""),"",IF(B18="Activity",D18*(E18/100)*(1+N(F18)+N(G18)),D18*(E18/100)*H18))</f>
+        <f>IF(OR(A18="",B18=""),"",IF(B18="Activity",MAX(0,N(D18))*(MIN(100,MAX(0,N(E18)))/100)*(1+MAX(0,N(F18))+MAX(0,N(G18))),MAX(0,N(D18))*(MIN(100,MAX(0,N(E18)))/100)*H18))</f>
         <v/>
       </c>
     </row>
@@ -2763,7 +2780,7 @@
         <v/>
       </c>
       <c r="I19" s="22">
-        <f>IF(OR(A19="",B19=""),"",IF(B19="Activity",D19*(E19/100)*(1+N(F19)+N(G19)),D19*(E19/100)*H19))</f>
+        <f>IF(OR(A19="",B19=""),"",IF(B19="Activity",MAX(0,N(D19))*(MIN(100,MAX(0,N(E19)))/100)*(1+MAX(0,N(F19))+MAX(0,N(G19))),MAX(0,N(D19))*(MIN(100,MAX(0,N(E19)))/100)*H19))</f>
         <v/>
       </c>
     </row>
@@ -2780,7 +2797,7 @@
         <v/>
       </c>
       <c r="I20" s="22">
-        <f>IF(OR(A20="",B20=""),"",IF(B20="Activity",D20*(E20/100)*(1+N(F20)+N(G20)),D20*(E20/100)*H20))</f>
+        <f>IF(OR(A20="",B20=""),"",IF(B20="Activity",MAX(0,N(D20))*(MIN(100,MAX(0,N(E20)))/100)*(1+MAX(0,N(F20))+MAX(0,N(G20))),MAX(0,N(D20))*(MIN(100,MAX(0,N(E20)))/100)*H20))</f>
         <v/>
       </c>
     </row>
@@ -2797,7 +2814,7 @@
         <v/>
       </c>
       <c r="I21" s="22">
-        <f>IF(OR(A21="",B21=""),"",IF(B21="Activity",D21*(E21/100)*(1+N(F21)+N(G21)),D21*(E21/100)*H21))</f>
+        <f>IF(OR(A21="",B21=""),"",IF(B21="Activity",MAX(0,N(D21))*(MIN(100,MAX(0,N(E21)))/100)*(1+MAX(0,N(F21))+MAX(0,N(G21))),MAX(0,N(D21))*(MIN(100,MAX(0,N(E21)))/100)*H21))</f>
         <v/>
       </c>
     </row>
@@ -2814,7 +2831,7 @@
         <v/>
       </c>
       <c r="I22" s="22">
-        <f>IF(OR(A22="",B22=""),"",IF(B22="Activity",D22*(E22/100)*(1+N(F22)+N(G22)),D22*(E22/100)*H22))</f>
+        <f>IF(OR(A22="",B22=""),"",IF(B22="Activity",MAX(0,N(D22))*(MIN(100,MAX(0,N(E22)))/100)*(1+MAX(0,N(F22))+MAX(0,N(G22))),MAX(0,N(D22))*(MIN(100,MAX(0,N(E22)))/100)*H22))</f>
         <v/>
       </c>
     </row>
@@ -2831,7 +2848,7 @@
         <v/>
       </c>
       <c r="I23" s="22">
-        <f>IF(OR(A23="",B23=""),"",IF(B23="Activity",D23*(E23/100)*(1+N(F23)+N(G23)),D23*(E23/100)*H23))</f>
+        <f>IF(OR(A23="",B23=""),"",IF(B23="Activity",MAX(0,N(D23))*(MIN(100,MAX(0,N(E23)))/100)*(1+MAX(0,N(F23))+MAX(0,N(G23))),MAX(0,N(D23))*(MIN(100,MAX(0,N(E23)))/100)*H23))</f>
         <v/>
       </c>
     </row>
@@ -2848,7 +2865,7 @@
         <v/>
       </c>
       <c r="I24" s="22">
-        <f>IF(OR(A24="",B24=""),"",IF(B24="Activity",D24*(E24/100)*(1+N(F24)+N(G24)),D24*(E24/100)*H24))</f>
+        <f>IF(OR(A24="",B24=""),"",IF(B24="Activity",MAX(0,N(D24))*(MIN(100,MAX(0,N(E24)))/100)*(1+MAX(0,N(F24))+MAX(0,N(G24))),MAX(0,N(D24))*(MIN(100,MAX(0,N(E24)))/100)*H24))</f>
         <v/>
       </c>
     </row>
@@ -2865,7 +2882,7 @@
         <v/>
       </c>
       <c r="I25" s="22">
-        <f>IF(OR(A25="",B25=""),"",IF(B25="Activity",D25*(E25/100)*(1+N(F25)+N(G25)),D25*(E25/100)*H25))</f>
+        <f>IF(OR(A25="",B25=""),"",IF(B25="Activity",MAX(0,N(D25))*(MIN(100,MAX(0,N(E25)))/100)*(1+MAX(0,N(F25))+MAX(0,N(G25))),MAX(0,N(D25))*(MIN(100,MAX(0,N(E25)))/100)*H25))</f>
         <v/>
       </c>
     </row>
@@ -2882,7 +2899,7 @@
         <v/>
       </c>
       <c r="I26" s="22">
-        <f>IF(OR(A26="",B26=""),"",IF(B26="Activity",D26*(E26/100)*(1+N(F26)+N(G26)),D26*(E26/100)*H26))</f>
+        <f>IF(OR(A26="",B26=""),"",IF(B26="Activity",MAX(0,N(D26))*(MIN(100,MAX(0,N(E26)))/100)*(1+MAX(0,N(F26))+MAX(0,N(G26))),MAX(0,N(D26))*(MIN(100,MAX(0,N(E26)))/100)*H26))</f>
         <v/>
       </c>
     </row>
@@ -2899,7 +2916,7 @@
         <v/>
       </c>
       <c r="I27" s="22">
-        <f>IF(OR(A27="",B27=""),"",IF(B27="Activity",D27*(E27/100)*(1+N(F27)+N(G27)),D27*(E27/100)*H27))</f>
+        <f>IF(OR(A27="",B27=""),"",IF(B27="Activity",MAX(0,N(D27))*(MIN(100,MAX(0,N(E27)))/100)*(1+MAX(0,N(F27))+MAX(0,N(G27))),MAX(0,N(D27))*(MIN(100,MAX(0,N(E27)))/100)*H27))</f>
         <v/>
       </c>
     </row>
@@ -2916,7 +2933,7 @@
         <v/>
       </c>
       <c r="I28" s="22">
-        <f>IF(OR(A28="",B28=""),"",IF(B28="Activity",D28*(E28/100)*(1+N(F28)+N(G28)),D28*(E28/100)*H28))</f>
+        <f>IF(OR(A28="",B28=""),"",IF(B28="Activity",MAX(0,N(D28))*(MIN(100,MAX(0,N(E28)))/100)*(1+MAX(0,N(F28))+MAX(0,N(G28))),MAX(0,N(D28))*(MIN(100,MAX(0,N(E28)))/100)*H28))</f>
         <v/>
       </c>
     </row>
@@ -2933,7 +2950,7 @@
         <v/>
       </c>
       <c r="I29" s="22">
-        <f>IF(OR(A29="",B29=""),"",IF(B29="Activity",D29*(E29/100)*(1+N(F29)+N(G29)),D29*(E29/100)*H29))</f>
+        <f>IF(OR(A29="",B29=""),"",IF(B29="Activity",MAX(0,N(D29))*(MIN(100,MAX(0,N(E29)))/100)*(1+MAX(0,N(F29))+MAX(0,N(G29))),MAX(0,N(D29))*(MIN(100,MAX(0,N(E29)))/100)*H29))</f>
         <v/>
       </c>
     </row>
@@ -2950,7 +2967,7 @@
         <v/>
       </c>
       <c r="I30" s="22">
-        <f>IF(OR(A30="",B30=""),"",IF(B30="Activity",D30*(E30/100)*(1+N(F30)+N(G30)),D30*(E30/100)*H30))</f>
+        <f>IF(OR(A30="",B30=""),"",IF(B30="Activity",MAX(0,N(D30))*(MIN(100,MAX(0,N(E30)))/100)*(1+MAX(0,N(F30))+MAX(0,N(G30))),MAX(0,N(D30))*(MIN(100,MAX(0,N(E30)))/100)*H30))</f>
         <v/>
       </c>
     </row>
@@ -2967,7 +2984,7 @@
         <v/>
       </c>
       <c r="I31" s="22">
-        <f>IF(OR(A31="",B31=""),"",IF(B31="Activity",D31*(E31/100)*(1+N(F31)+N(G31)),D31*(E31/100)*H31))</f>
+        <f>IF(OR(A31="",B31=""),"",IF(B31="Activity",MAX(0,N(D31))*(MIN(100,MAX(0,N(E31)))/100)*(1+MAX(0,N(F31))+MAX(0,N(G31))),MAX(0,N(D31))*(MIN(100,MAX(0,N(E31)))/100)*H31))</f>
         <v/>
       </c>
     </row>
@@ -2984,7 +3001,7 @@
         <v/>
       </c>
       <c r="I32" s="22">
-        <f>IF(OR(A32="",B32=""),"",IF(B32="Activity",D32*(E32/100)*(1+N(F32)+N(G32)),D32*(E32/100)*H32))</f>
+        <f>IF(OR(A32="",B32=""),"",IF(B32="Activity",MAX(0,N(D32))*(MIN(100,MAX(0,N(E32)))/100)*(1+MAX(0,N(F32))+MAX(0,N(G32))),MAX(0,N(D32))*(MIN(100,MAX(0,N(E32)))/100)*H32))</f>
         <v/>
       </c>
     </row>
@@ -3001,7 +3018,7 @@
         <v/>
       </c>
       <c r="I33" s="22">
-        <f>IF(OR(A33="",B33=""),"",IF(B33="Activity",D33*(E33/100)*(1+N(F33)+N(G33)),D33*(E33/100)*H33))</f>
+        <f>IF(OR(A33="",B33=""),"",IF(B33="Activity",MAX(0,N(D33))*(MIN(100,MAX(0,N(E33)))/100)*(1+MAX(0,N(F33))+MAX(0,N(G33))),MAX(0,N(D33))*(MIN(100,MAX(0,N(E33)))/100)*H33))</f>
         <v/>
       </c>
     </row>
@@ -3018,7 +3035,7 @@
         <v/>
       </c>
       <c r="I34" s="22">
-        <f>IF(OR(A34="",B34=""),"",IF(B34="Activity",D34*(E34/100)*(1+N(F34)+N(G34)),D34*(E34/100)*H34))</f>
+        <f>IF(OR(A34="",B34=""),"",IF(B34="Activity",MAX(0,N(D34))*(MIN(100,MAX(0,N(E34)))/100)*(1+MAX(0,N(F34))+MAX(0,N(G34))),MAX(0,N(D34))*(MIN(100,MAX(0,N(E34)))/100)*H34))</f>
         <v/>
       </c>
     </row>
@@ -3035,7 +3052,7 @@
         <v/>
       </c>
       <c r="I35" s="22">
-        <f>IF(OR(A35="",B35=""),"",IF(B35="Activity",D35*(E35/100)*(1+N(F35)+N(G35)),D35*(E35/100)*H35))</f>
+        <f>IF(OR(A35="",B35=""),"",IF(B35="Activity",MAX(0,N(D35))*(MIN(100,MAX(0,N(E35)))/100)*(1+MAX(0,N(F35))+MAX(0,N(G35))),MAX(0,N(D35))*(MIN(100,MAX(0,N(E35)))/100)*H35))</f>
         <v/>
       </c>
     </row>
@@ -3052,7 +3069,7 @@
         <v/>
       </c>
       <c r="I36" s="22">
-        <f>IF(OR(A36="",B36=""),"",IF(B36="Activity",D36*(E36/100)*(1+N(F36)+N(G36)),D36*(E36/100)*H36))</f>
+        <f>IF(OR(A36="",B36=""),"",IF(B36="Activity",MAX(0,N(D36))*(MIN(100,MAX(0,N(E36)))/100)*(1+MAX(0,N(F36))+MAX(0,N(G36))),MAX(0,N(D36))*(MIN(100,MAX(0,N(E36)))/100)*H36))</f>
         <v/>
       </c>
     </row>
@@ -3069,7 +3086,7 @@
         <v/>
       </c>
       <c r="I37" s="22">
-        <f>IF(OR(A37="",B37=""),"",IF(B37="Activity",D37*(E37/100)*(1+N(F37)+N(G37)),D37*(E37/100)*H37))</f>
+        <f>IF(OR(A37="",B37=""),"",IF(B37="Activity",MAX(0,N(D37))*(MIN(100,MAX(0,N(E37)))/100)*(1+MAX(0,N(F37))+MAX(0,N(G37))),MAX(0,N(D37))*(MIN(100,MAX(0,N(E37)))/100)*H37))</f>
         <v/>
       </c>
     </row>
@@ -3086,7 +3103,7 @@
         <v/>
       </c>
       <c r="I38" s="22">
-        <f>IF(OR(A38="",B38=""),"",IF(B38="Activity",D38*(E38/100)*(1+N(F38)+N(G38)),D38*(E38/100)*H38))</f>
+        <f>IF(OR(A38="",B38=""),"",IF(B38="Activity",MAX(0,N(D38))*(MIN(100,MAX(0,N(E38)))/100)*(1+MAX(0,N(F38))+MAX(0,N(G38))),MAX(0,N(D38))*(MIN(100,MAX(0,N(E38)))/100)*H38))</f>
         <v/>
       </c>
     </row>
@@ -3103,7 +3120,7 @@
         <v/>
       </c>
       <c r="I39" s="22">
-        <f>IF(OR(A39="",B39=""),"",IF(B39="Activity",D39*(E39/100)*(1+N(F39)+N(G39)),D39*(E39/100)*H39))</f>
+        <f>IF(OR(A39="",B39=""),"",IF(B39="Activity",MAX(0,N(D39))*(MIN(100,MAX(0,N(E39)))/100)*(1+MAX(0,N(F39))+MAX(0,N(G39))),MAX(0,N(D39))*(MIN(100,MAX(0,N(E39)))/100)*H39))</f>
         <v/>
       </c>
     </row>
@@ -3120,7 +3137,7 @@
         <v/>
       </c>
       <c r="I40" s="22">
-        <f>IF(OR(A40="",B40=""),"",IF(B40="Activity",D40*(E40/100)*(1+N(F40)+N(G40)),D40*(E40/100)*H40))</f>
+        <f>IF(OR(A40="",B40=""),"",IF(B40="Activity",MAX(0,N(D40))*(MIN(100,MAX(0,N(E40)))/100)*(1+MAX(0,N(F40))+MAX(0,N(G40))),MAX(0,N(D40))*(MIN(100,MAX(0,N(E40)))/100)*H40))</f>
         <v/>
       </c>
     </row>
@@ -3137,7 +3154,7 @@
         <v/>
       </c>
       <c r="I41" s="22">
-        <f>IF(OR(A41="",B41=""),"",IF(B41="Activity",D41*(E41/100)*(1+N(F41)+N(G41)),D41*(E41/100)*H41))</f>
+        <f>IF(OR(A41="",B41=""),"",IF(B41="Activity",MAX(0,N(D41))*(MIN(100,MAX(0,N(E41)))/100)*(1+MAX(0,N(F41))+MAX(0,N(G41))),MAX(0,N(D41))*(MIN(100,MAX(0,N(E41)))/100)*H41))</f>
         <v/>
       </c>
     </row>
@@ -3154,7 +3171,7 @@
         <v/>
       </c>
       <c r="I42" s="22">
-        <f>IF(OR(A42="",B42=""),"",IF(B42="Activity",D42*(E42/100)*(1+N(F42)+N(G42)),D42*(E42/100)*H42))</f>
+        <f>IF(OR(A42="",B42=""),"",IF(B42="Activity",MAX(0,N(D42))*(MIN(100,MAX(0,N(E42)))/100)*(1+MAX(0,N(F42))+MAX(0,N(G42))),MAX(0,N(D42))*(MIN(100,MAX(0,N(E42)))/100)*H42))</f>
         <v/>
       </c>
     </row>
@@ -3171,7 +3188,7 @@
         <v/>
       </c>
       <c r="I43" s="22">
-        <f>IF(OR(A43="",B43=""),"",IF(B43="Activity",D43*(E43/100)*(1+N(F43)+N(G43)),D43*(E43/100)*H43))</f>
+        <f>IF(OR(A43="",B43=""),"",IF(B43="Activity",MAX(0,N(D43))*(MIN(100,MAX(0,N(E43)))/100)*(1+MAX(0,N(F43))+MAX(0,N(G43))),MAX(0,N(D43))*(MIN(100,MAX(0,N(E43)))/100)*H43))</f>
         <v/>
       </c>
     </row>
@@ -3188,7 +3205,7 @@
         <v/>
       </c>
       <c r="I44" s="22">
-        <f>IF(OR(A44="",B44=""),"",IF(B44="Activity",D44*(E44/100)*(1+N(F44)+N(G44)),D44*(E44/100)*H44))</f>
+        <f>IF(OR(A44="",B44=""),"",IF(B44="Activity",MAX(0,N(D44))*(MIN(100,MAX(0,N(E44)))/100)*(1+MAX(0,N(F44))+MAX(0,N(G44))),MAX(0,N(D44))*(MIN(100,MAX(0,N(E44)))/100)*H44))</f>
         <v/>
       </c>
     </row>
@@ -3205,7 +3222,7 @@
         <v/>
       </c>
       <c r="I45" s="22">
-        <f>IF(OR(A45="",B45=""),"",IF(B45="Activity",D45*(E45/100)*(1+N(F45)+N(G45)),D45*(E45/100)*H45))</f>
+        <f>IF(OR(A45="",B45=""),"",IF(B45="Activity",MAX(0,N(D45))*(MIN(100,MAX(0,N(E45)))/100)*(1+MAX(0,N(F45))+MAX(0,N(G45))),MAX(0,N(D45))*(MIN(100,MAX(0,N(E45)))/100)*H45))</f>
         <v/>
       </c>
     </row>
@@ -3222,7 +3239,7 @@
         <v/>
       </c>
       <c r="I46" s="22">
-        <f>IF(OR(A46="",B46=""),"",IF(B46="Activity",D46*(E46/100)*(1+N(F46)+N(G46)),D46*(E46/100)*H46))</f>
+        <f>IF(OR(A46="",B46=""),"",IF(B46="Activity",MAX(0,N(D46))*(MIN(100,MAX(0,N(E46)))/100)*(1+MAX(0,N(F46))+MAX(0,N(G46))),MAX(0,N(D46))*(MIN(100,MAX(0,N(E46)))/100)*H46))</f>
         <v/>
       </c>
     </row>
@@ -3239,7 +3256,7 @@
         <v/>
       </c>
       <c r="I47" s="22">
-        <f>IF(OR(A47="",B47=""),"",IF(B47="Activity",D47*(E47/100)*(1+N(F47)+N(G47)),D47*(E47/100)*H47))</f>
+        <f>IF(OR(A47="",B47=""),"",IF(B47="Activity",MAX(0,N(D47))*(MIN(100,MAX(0,N(E47)))/100)*(1+MAX(0,N(F47))+MAX(0,N(G47))),MAX(0,N(D47))*(MIN(100,MAX(0,N(E47)))/100)*H47))</f>
         <v/>
       </c>
     </row>
@@ -3256,7 +3273,7 @@
         <v/>
       </c>
       <c r="I48" s="22">
-        <f>IF(OR(A48="",B48=""),"",IF(B48="Activity",D48*(E48/100)*(1+N(F48)+N(G48)),D48*(E48/100)*H48))</f>
+        <f>IF(OR(A48="",B48=""),"",IF(B48="Activity",MAX(0,N(D48))*(MIN(100,MAX(0,N(E48)))/100)*(1+MAX(0,N(F48))+MAX(0,N(G48))),MAX(0,N(D48))*(MIN(100,MAX(0,N(E48)))/100)*H48))</f>
         <v/>
       </c>
     </row>
@@ -3273,7 +3290,7 @@
         <v/>
       </c>
       <c r="I49" s="22">
-        <f>IF(OR(A49="",B49=""),"",IF(B49="Activity",D49*(E49/100)*(1+N(F49)+N(G49)),D49*(E49/100)*H49))</f>
+        <f>IF(OR(A49="",B49=""),"",IF(B49="Activity",MAX(0,N(D49))*(MIN(100,MAX(0,N(E49)))/100)*(1+MAX(0,N(F49))+MAX(0,N(G49))),MAX(0,N(D49))*(MIN(100,MAX(0,N(E49)))/100)*H49))</f>
         <v/>
       </c>
     </row>
@@ -3290,7 +3307,7 @@
         <v/>
       </c>
       <c r="I50" s="22">
-        <f>IF(OR(A50="",B50=""),"",IF(B50="Activity",D50*(E50/100)*(1+N(F50)+N(G50)),D50*(E50/100)*H50))</f>
+        <f>IF(OR(A50="",B50=""),"",IF(B50="Activity",MAX(0,N(D50))*(MIN(100,MAX(0,N(E50)))/100)*(1+MAX(0,N(F50))+MAX(0,N(G50))),MAX(0,N(D50))*(MIN(100,MAX(0,N(E50)))/100)*H50))</f>
         <v/>
       </c>
     </row>
@@ -3307,7 +3324,7 @@
         <v/>
       </c>
       <c r="I51" s="22">
-        <f>IF(OR(A51="",B51=""),"",IF(B51="Activity",D51*(E51/100)*(1+N(F51)+N(G51)),D51*(E51/100)*H51))</f>
+        <f>IF(OR(A51="",B51=""),"",IF(B51="Activity",MAX(0,N(D51))*(MIN(100,MAX(0,N(E51)))/100)*(1+MAX(0,N(F51))+MAX(0,N(G51))),MAX(0,N(D51))*(MIN(100,MAX(0,N(E51)))/100)*H51))</f>
         <v/>
       </c>
     </row>
@@ -3324,7 +3341,7 @@
         <v/>
       </c>
       <c r="I52" s="22">
-        <f>IF(OR(A52="",B52=""),"",IF(B52="Activity",D52*(E52/100)*(1+N(F52)+N(G52)),D52*(E52/100)*H52))</f>
+        <f>IF(OR(A52="",B52=""),"",IF(B52="Activity",MAX(0,N(D52))*(MIN(100,MAX(0,N(E52)))/100)*(1+MAX(0,N(F52))+MAX(0,N(G52))),MAX(0,N(D52))*(MIN(100,MAX(0,N(E52)))/100)*H52))</f>
         <v/>
       </c>
     </row>
@@ -3341,7 +3358,7 @@
         <v/>
       </c>
       <c r="I53" s="22">
-        <f>IF(OR(A53="",B53=""),"",IF(B53="Activity",D53*(E53/100)*(1+N(F53)+N(G53)),D53*(E53/100)*H53))</f>
+        <f>IF(OR(A53="",B53=""),"",IF(B53="Activity",MAX(0,N(D53))*(MIN(100,MAX(0,N(E53)))/100)*(1+MAX(0,N(F53))+MAX(0,N(G53))),MAX(0,N(D53))*(MIN(100,MAX(0,N(E53)))/100)*H53))</f>
         <v/>
       </c>
     </row>
@@ -3358,7 +3375,7 @@
         <v/>
       </c>
       <c r="I54" s="22">
-        <f>IF(OR(A54="",B54=""),"",IF(B54="Activity",D54*(E54/100)*(1+N(F54)+N(G54)),D54*(E54/100)*H54))</f>
+        <f>IF(OR(A54="",B54=""),"",IF(B54="Activity",MAX(0,N(D54))*(MIN(100,MAX(0,N(E54)))/100)*(1+MAX(0,N(F54))+MAX(0,N(G54))),MAX(0,N(D54))*(MIN(100,MAX(0,N(E54)))/100)*H54))</f>
         <v/>
       </c>
     </row>
@@ -3375,7 +3392,7 @@
         <v/>
       </c>
       <c r="I55" s="22">
-        <f>IF(OR(A55="",B55=""),"",IF(B55="Activity",D55*(E55/100)*(1+N(F55)+N(G55)),D55*(E55/100)*H55))</f>
+        <f>IF(OR(A55="",B55=""),"",IF(B55="Activity",MAX(0,N(D55))*(MIN(100,MAX(0,N(E55)))/100)*(1+MAX(0,N(F55))+MAX(0,N(G55))),MAX(0,N(D55))*(MIN(100,MAX(0,N(E55)))/100)*H55))</f>
         <v/>
       </c>
     </row>
@@ -3392,7 +3409,7 @@
         <v/>
       </c>
       <c r="I56" s="22">
-        <f>IF(OR(A56="",B56=""),"",IF(B56="Activity",D56*(E56/100)*(1+N(F56)+N(G56)),D56*(E56/100)*H56))</f>
+        <f>IF(OR(A56="",B56=""),"",IF(B56="Activity",MAX(0,N(D56))*(MIN(100,MAX(0,N(E56)))/100)*(1+MAX(0,N(F56))+MAX(0,N(G56))),MAX(0,N(D56))*(MIN(100,MAX(0,N(E56)))/100)*H56))</f>
         <v/>
       </c>
     </row>
@@ -3409,7 +3426,7 @@
         <v/>
       </c>
       <c r="I57" s="22">
-        <f>IF(OR(A57="",B57=""),"",IF(B57="Activity",D57*(E57/100)*(1+N(F57)+N(G57)),D57*(E57/100)*H57))</f>
+        <f>IF(OR(A57="",B57=""),"",IF(B57="Activity",MAX(0,N(D57))*(MIN(100,MAX(0,N(E57)))/100)*(1+MAX(0,N(F57))+MAX(0,N(G57))),MAX(0,N(D57))*(MIN(100,MAX(0,N(E57)))/100)*H57))</f>
         <v/>
       </c>
     </row>
@@ -3426,7 +3443,7 @@
         <v/>
       </c>
       <c r="I58" s="22">
-        <f>IF(OR(A58="",B58=""),"",IF(B58="Activity",D58*(E58/100)*(1+N(F58)+N(G58)),D58*(E58/100)*H58))</f>
+        <f>IF(OR(A58="",B58=""),"",IF(B58="Activity",MAX(0,N(D58))*(MIN(100,MAX(0,N(E58)))/100)*(1+MAX(0,N(F58))+MAX(0,N(G58))),MAX(0,N(D58))*(MIN(100,MAX(0,N(E58)))/100)*H58))</f>
         <v/>
       </c>
     </row>
@@ -3443,7 +3460,7 @@
         <v/>
       </c>
       <c r="I59" s="22">
-        <f>IF(OR(A59="",B59=""),"",IF(B59="Activity",D59*(E59/100)*(1+N(F59)+N(G59)),D59*(E59/100)*H59))</f>
+        <f>IF(OR(A59="",B59=""),"",IF(B59="Activity",MAX(0,N(D59))*(MIN(100,MAX(0,N(E59)))/100)*(1+MAX(0,N(F59))+MAX(0,N(G59))),MAX(0,N(D59))*(MIN(100,MAX(0,N(E59)))/100)*H59))</f>
         <v/>
       </c>
     </row>
@@ -3460,7 +3477,7 @@
         <v/>
       </c>
       <c r="I60" s="22">
-        <f>IF(OR(A60="",B60=""),"",IF(B60="Activity",D60*(E60/100)*(1+N(F60)+N(G60)),D60*(E60/100)*H60))</f>
+        <f>IF(OR(A60="",B60=""),"",IF(B60="Activity",MAX(0,N(D60))*(MIN(100,MAX(0,N(E60)))/100)*(1+MAX(0,N(F60))+MAX(0,N(G60))),MAX(0,N(D60))*(MIN(100,MAX(0,N(E60)))/100)*H60))</f>
         <v/>
       </c>
     </row>
@@ -3477,7 +3494,7 @@
         <v/>
       </c>
       <c r="I61" s="22">
-        <f>IF(OR(A61="",B61=""),"",IF(B61="Activity",D61*(E61/100)*(1+N(F61)+N(G61)),D61*(E61/100)*H61))</f>
+        <f>IF(OR(A61="",B61=""),"",IF(B61="Activity",MAX(0,N(D61))*(MIN(100,MAX(0,N(E61)))/100)*(1+MAX(0,N(F61))+MAX(0,N(G61))),MAX(0,N(D61))*(MIN(100,MAX(0,N(E61)))/100)*H61))</f>
         <v/>
       </c>
     </row>
@@ -3494,7 +3511,7 @@
         <v/>
       </c>
       <c r="I62" s="22">
-        <f>IF(OR(A62="",B62=""),"",IF(B62="Activity",D62*(E62/100)*(1+N(F62)+N(G62)),D62*(E62/100)*H62))</f>
+        <f>IF(OR(A62="",B62=""),"",IF(B62="Activity",MAX(0,N(D62))*(MIN(100,MAX(0,N(E62)))/100)*(1+MAX(0,N(F62))+MAX(0,N(G62))),MAX(0,N(D62))*(MIN(100,MAX(0,N(E62)))/100)*H62))</f>
         <v/>
       </c>
     </row>
@@ -3511,7 +3528,7 @@
         <v/>
       </c>
       <c r="I63" s="22">
-        <f>IF(OR(A63="",B63=""),"",IF(B63="Activity",D63*(E63/100)*(1+N(F63)+N(G63)),D63*(E63/100)*H63))</f>
+        <f>IF(OR(A63="",B63=""),"",IF(B63="Activity",MAX(0,N(D63))*(MIN(100,MAX(0,N(E63)))/100)*(1+MAX(0,N(F63))+MAX(0,N(G63))),MAX(0,N(D63))*(MIN(100,MAX(0,N(E63)))/100)*H63))</f>
         <v/>
       </c>
     </row>
@@ -3528,7 +3545,7 @@
         <v/>
       </c>
       <c r="I64" s="22">
-        <f>IF(OR(A64="",B64=""),"",IF(B64="Activity",D64*(E64/100)*(1+N(F64)+N(G64)),D64*(E64/100)*H64))</f>
+        <f>IF(OR(A64="",B64=""),"",IF(B64="Activity",MAX(0,N(D64))*(MIN(100,MAX(0,N(E64)))/100)*(1+MAX(0,N(F64))+MAX(0,N(G64))),MAX(0,N(D64))*(MIN(100,MAX(0,N(E64)))/100)*H64))</f>
         <v/>
       </c>
     </row>
@@ -3545,7 +3562,7 @@
         <v/>
       </c>
       <c r="I65" s="22">
-        <f>IF(OR(A65="",B65=""),"",IF(B65="Activity",D65*(E65/100)*(1+N(F65)+N(G65)),D65*(E65/100)*H65))</f>
+        <f>IF(OR(A65="",B65=""),"",IF(B65="Activity",MAX(0,N(D65))*(MIN(100,MAX(0,N(E65)))/100)*(1+MAX(0,N(F65))+MAX(0,N(G65))),MAX(0,N(D65))*(MIN(100,MAX(0,N(E65)))/100)*H65))</f>
         <v/>
       </c>
     </row>
@@ -3562,7 +3579,7 @@
         <v/>
       </c>
       <c r="I66" s="22">
-        <f>IF(OR(A66="",B66=""),"",IF(B66="Activity",D66*(E66/100)*(1+N(F66)+N(G66)),D66*(E66/100)*H66))</f>
+        <f>IF(OR(A66="",B66=""),"",IF(B66="Activity",MAX(0,N(D66))*(MIN(100,MAX(0,N(E66)))/100)*(1+MAX(0,N(F66))+MAX(0,N(G66))),MAX(0,N(D66))*(MIN(100,MAX(0,N(E66)))/100)*H66))</f>
         <v/>
       </c>
     </row>
@@ -3579,7 +3596,7 @@
         <v/>
       </c>
       <c r="I67" s="22">
-        <f>IF(OR(A67="",B67=""),"",IF(B67="Activity",D67*(E67/100)*(1+N(F67)+N(G67)),D67*(E67/100)*H67))</f>
+        <f>IF(OR(A67="",B67=""),"",IF(B67="Activity",MAX(0,N(D67))*(MIN(100,MAX(0,N(E67)))/100)*(1+MAX(0,N(F67))+MAX(0,N(G67))),MAX(0,N(D67))*(MIN(100,MAX(0,N(E67)))/100)*H67))</f>
         <v/>
       </c>
     </row>
@@ -3596,7 +3613,7 @@
         <v/>
       </c>
       <c r="I68" s="22">
-        <f>IF(OR(A68="",B68=""),"",IF(B68="Activity",D68*(E68/100)*(1+N(F68)+N(G68)),D68*(E68/100)*H68))</f>
+        <f>IF(OR(A68="",B68=""),"",IF(B68="Activity",MAX(0,N(D68))*(MIN(100,MAX(0,N(E68)))/100)*(1+MAX(0,N(F68))+MAX(0,N(G68))),MAX(0,N(D68))*(MIN(100,MAX(0,N(E68)))/100)*H68))</f>
         <v/>
       </c>
     </row>
@@ -3613,7 +3630,7 @@
         <v/>
       </c>
       <c r="I69" s="22">
-        <f>IF(OR(A69="",B69=""),"",IF(B69="Activity",D69*(E69/100)*(1+N(F69)+N(G69)),D69*(E69/100)*H69))</f>
+        <f>IF(OR(A69="",B69=""),"",IF(B69="Activity",MAX(0,N(D69))*(MIN(100,MAX(0,N(E69)))/100)*(1+MAX(0,N(F69))+MAX(0,N(G69))),MAX(0,N(D69))*(MIN(100,MAX(0,N(E69)))/100)*H69))</f>
         <v/>
       </c>
     </row>
@@ -3630,7 +3647,7 @@
         <v/>
       </c>
       <c r="I70" s="22">
-        <f>IF(OR(A70="",B70=""),"",IF(B70="Activity",D70*(E70/100)*(1+N(F70)+N(G70)),D70*(E70/100)*H70))</f>
+        <f>IF(OR(A70="",B70=""),"",IF(B70="Activity",MAX(0,N(D70))*(MIN(100,MAX(0,N(E70)))/100)*(1+MAX(0,N(F70))+MAX(0,N(G70))),MAX(0,N(D70))*(MIN(100,MAX(0,N(E70)))/100)*H70))</f>
         <v/>
       </c>
     </row>
@@ -3647,7 +3664,7 @@
         <v/>
       </c>
       <c r="I71" s="22">
-        <f>IF(OR(A71="",B71=""),"",IF(B71="Activity",D71*(E71/100)*(1+N(F71)+N(G71)),D71*(E71/100)*H71))</f>
+        <f>IF(OR(A71="",B71=""),"",IF(B71="Activity",MAX(0,N(D71))*(MIN(100,MAX(0,N(E71)))/100)*(1+MAX(0,N(F71))+MAX(0,N(G71))),MAX(0,N(D71))*(MIN(100,MAX(0,N(E71)))/100)*H71))</f>
         <v/>
       </c>
     </row>
@@ -3664,7 +3681,7 @@
         <v/>
       </c>
       <c r="I72" s="22">
-        <f>IF(OR(A72="",B72=""),"",IF(B72="Activity",D72*(E72/100)*(1+N(F72)+N(G72)),D72*(E72/100)*H72))</f>
+        <f>IF(OR(A72="",B72=""),"",IF(B72="Activity",MAX(0,N(D72))*(MIN(100,MAX(0,N(E72)))/100)*(1+MAX(0,N(F72))+MAX(0,N(G72))),MAX(0,N(D72))*(MIN(100,MAX(0,N(E72)))/100)*H72))</f>
         <v/>
       </c>
     </row>
@@ -3681,7 +3698,7 @@
         <v/>
       </c>
       <c r="I73" s="22">
-        <f>IF(OR(A73="",B73=""),"",IF(B73="Activity",D73*(E73/100)*(1+N(F73)+N(G73)),D73*(E73/100)*H73))</f>
+        <f>IF(OR(A73="",B73=""),"",IF(B73="Activity",MAX(0,N(D73))*(MIN(100,MAX(0,N(E73)))/100)*(1+MAX(0,N(F73))+MAX(0,N(G73))),MAX(0,N(D73))*(MIN(100,MAX(0,N(E73)))/100)*H73))</f>
         <v/>
       </c>
     </row>
@@ -3698,7 +3715,7 @@
         <v/>
       </c>
       <c r="I74" s="22">
-        <f>IF(OR(A74="",B74=""),"",IF(B74="Activity",D74*(E74/100)*(1+N(F74)+N(G74)),D74*(E74/100)*H74))</f>
+        <f>IF(OR(A74="",B74=""),"",IF(B74="Activity",MAX(0,N(D74))*(MIN(100,MAX(0,N(E74)))/100)*(1+MAX(0,N(F74))+MAX(0,N(G74))),MAX(0,N(D74))*(MIN(100,MAX(0,N(E74)))/100)*H74))</f>
         <v/>
       </c>
     </row>
@@ -3715,7 +3732,7 @@
         <v/>
       </c>
       <c r="I75" s="22">
-        <f>IF(OR(A75="",B75=""),"",IF(B75="Activity",D75*(E75/100)*(1+N(F75)+N(G75)),D75*(E75/100)*H75))</f>
+        <f>IF(OR(A75="",B75=""),"",IF(B75="Activity",MAX(0,N(D75))*(MIN(100,MAX(0,N(E75)))/100)*(1+MAX(0,N(F75))+MAX(0,N(G75))),MAX(0,N(D75))*(MIN(100,MAX(0,N(E75)))/100)*H75))</f>
         <v/>
       </c>
     </row>
@@ -3732,7 +3749,7 @@
         <v/>
       </c>
       <c r="I76" s="22">
-        <f>IF(OR(A76="",B76=""),"",IF(B76="Activity",D76*(E76/100)*(1+N(F76)+N(G76)),D76*(E76/100)*H76))</f>
+        <f>IF(OR(A76="",B76=""),"",IF(B76="Activity",MAX(0,N(D76))*(MIN(100,MAX(0,N(E76)))/100)*(1+MAX(0,N(F76))+MAX(0,N(G76))),MAX(0,N(D76))*(MIN(100,MAX(0,N(E76)))/100)*H76))</f>
         <v/>
       </c>
     </row>
@@ -3749,7 +3766,7 @@
         <v/>
       </c>
       <c r="I77" s="22">
-        <f>IF(OR(A77="",B77=""),"",IF(B77="Activity",D77*(E77/100)*(1+N(F77)+N(G77)),D77*(E77/100)*H77))</f>
+        <f>IF(OR(A77="",B77=""),"",IF(B77="Activity",MAX(0,N(D77))*(MIN(100,MAX(0,N(E77)))/100)*(1+MAX(0,N(F77))+MAX(0,N(G77))),MAX(0,N(D77))*(MIN(100,MAX(0,N(E77)))/100)*H77))</f>
         <v/>
       </c>
     </row>
@@ -3766,7 +3783,7 @@
         <v/>
       </c>
       <c r="I78" s="22">
-        <f>IF(OR(A78="",B78=""),"",IF(B78="Activity",D78*(E78/100)*(1+N(F78)+N(G78)),D78*(E78/100)*H78))</f>
+        <f>IF(OR(A78="",B78=""),"",IF(B78="Activity",MAX(0,N(D78))*(MIN(100,MAX(0,N(E78)))/100)*(1+MAX(0,N(F78))+MAX(0,N(G78))),MAX(0,N(D78))*(MIN(100,MAX(0,N(E78)))/100)*H78))</f>
         <v/>
       </c>
     </row>
@@ -3783,7 +3800,7 @@
         <v/>
       </c>
       <c r="I79" s="22">
-        <f>IF(OR(A79="",B79=""),"",IF(B79="Activity",D79*(E79/100)*(1+N(F79)+N(G79)),D79*(E79/100)*H79))</f>
+        <f>IF(OR(A79="",B79=""),"",IF(B79="Activity",MAX(0,N(D79))*(MIN(100,MAX(0,N(E79)))/100)*(1+MAX(0,N(F79))+MAX(0,N(G79))),MAX(0,N(D79))*(MIN(100,MAX(0,N(E79)))/100)*H79))</f>
         <v/>
       </c>
     </row>
@@ -3800,7 +3817,7 @@
         <v/>
       </c>
       <c r="I80" s="22">
-        <f>IF(OR(A80="",B80=""),"",IF(B80="Activity",D80*(E80/100)*(1+N(F80)+N(G80)),D80*(E80/100)*H80))</f>
+        <f>IF(OR(A80="",B80=""),"",IF(B80="Activity",MAX(0,N(D80))*(MIN(100,MAX(0,N(E80)))/100)*(1+MAX(0,N(F80))+MAX(0,N(G80))),MAX(0,N(D80))*(MIN(100,MAX(0,N(E80)))/100)*H80))</f>
         <v/>
       </c>
     </row>
@@ -3817,7 +3834,7 @@
         <v/>
       </c>
       <c r="I81" s="22">
-        <f>IF(OR(A81="",B81=""),"",IF(B81="Activity",D81*(E81/100)*(1+N(F81)+N(G81)),D81*(E81/100)*H81))</f>
+        <f>IF(OR(A81="",B81=""),"",IF(B81="Activity",MAX(0,N(D81))*(MIN(100,MAX(0,N(E81)))/100)*(1+MAX(0,N(F81))+MAX(0,N(G81))),MAX(0,N(D81))*(MIN(100,MAX(0,N(E81)))/100)*H81))</f>
         <v/>
       </c>
     </row>
@@ -3834,7 +3851,7 @@
         <v/>
       </c>
       <c r="I82" s="22">
-        <f>IF(OR(A82="",B82=""),"",IF(B82="Activity",D82*(E82/100)*(1+N(F82)+N(G82)),D82*(E82/100)*H82))</f>
+        <f>IF(OR(A82="",B82=""),"",IF(B82="Activity",MAX(0,N(D82))*(MIN(100,MAX(0,N(E82)))/100)*(1+MAX(0,N(F82))+MAX(0,N(G82))),MAX(0,N(D82))*(MIN(100,MAX(0,N(E82)))/100)*H82))</f>
         <v/>
       </c>
     </row>
@@ -3851,7 +3868,7 @@
         <v/>
       </c>
       <c r="I83" s="22">
-        <f>IF(OR(A83="",B83=""),"",IF(B83="Activity",D83*(E83/100)*(1+N(F83)+N(G83)),D83*(E83/100)*H83))</f>
+        <f>IF(OR(A83="",B83=""),"",IF(B83="Activity",MAX(0,N(D83))*(MIN(100,MAX(0,N(E83)))/100)*(1+MAX(0,N(F83))+MAX(0,N(G83))),MAX(0,N(D83))*(MIN(100,MAX(0,N(E83)))/100)*H83))</f>
         <v/>
       </c>
     </row>
@@ -3868,7 +3885,7 @@
         <v/>
       </c>
       <c r="I84" s="22">
-        <f>IF(OR(A84="",B84=""),"",IF(B84="Activity",D84*(E84/100)*(1+N(F84)+N(G84)),D84*(E84/100)*H84))</f>
+        <f>IF(OR(A84="",B84=""),"",IF(B84="Activity",MAX(0,N(D84))*(MIN(100,MAX(0,N(E84)))/100)*(1+MAX(0,N(F84))+MAX(0,N(G84))),MAX(0,N(D84))*(MIN(100,MAX(0,N(E84)))/100)*H84))</f>
         <v/>
       </c>
     </row>
@@ -3885,7 +3902,7 @@
         <v/>
       </c>
       <c r="I85" s="22">
-        <f>IF(OR(A85="",B85=""),"",IF(B85="Activity",D85*(E85/100)*(1+N(F85)+N(G85)),D85*(E85/100)*H85))</f>
+        <f>IF(OR(A85="",B85=""),"",IF(B85="Activity",MAX(0,N(D85))*(MIN(100,MAX(0,N(E85)))/100)*(1+MAX(0,N(F85))+MAX(0,N(G85))),MAX(0,N(D85))*(MIN(100,MAX(0,N(E85)))/100)*H85))</f>
         <v/>
       </c>
     </row>
@@ -3902,7 +3919,7 @@
         <v/>
       </c>
       <c r="I86" s="22">
-        <f>IF(OR(A86="",B86=""),"",IF(B86="Activity",D86*(E86/100)*(1+N(F86)+N(G86)),D86*(E86/100)*H86))</f>
+        <f>IF(OR(A86="",B86=""),"",IF(B86="Activity",MAX(0,N(D86))*(MIN(100,MAX(0,N(E86)))/100)*(1+MAX(0,N(F86))+MAX(0,N(G86))),MAX(0,N(D86))*(MIN(100,MAX(0,N(E86)))/100)*H86))</f>
         <v/>
       </c>
     </row>
@@ -3919,7 +3936,7 @@
         <v/>
       </c>
       <c r="I87" s="22">
-        <f>IF(OR(A87="",B87=""),"",IF(B87="Activity",D87*(E87/100)*(1+N(F87)+N(G87)),D87*(E87/100)*H87))</f>
+        <f>IF(OR(A87="",B87=""),"",IF(B87="Activity",MAX(0,N(D87))*(MIN(100,MAX(0,N(E87)))/100)*(1+MAX(0,N(F87))+MAX(0,N(G87))),MAX(0,N(D87))*(MIN(100,MAX(0,N(E87)))/100)*H87))</f>
         <v/>
       </c>
     </row>
@@ -3936,7 +3953,7 @@
         <v/>
       </c>
       <c r="I88" s="22">
-        <f>IF(OR(A88="",B88=""),"",IF(B88="Activity",D88*(E88/100)*(1+N(F88)+N(G88)),D88*(E88/100)*H88))</f>
+        <f>IF(OR(A88="",B88=""),"",IF(B88="Activity",MAX(0,N(D88))*(MIN(100,MAX(0,N(E88)))/100)*(1+MAX(0,N(F88))+MAX(0,N(G88))),MAX(0,N(D88))*(MIN(100,MAX(0,N(E88)))/100)*H88))</f>
         <v/>
       </c>
     </row>
@@ -3953,7 +3970,7 @@
         <v/>
       </c>
       <c r="I89" s="22">
-        <f>IF(OR(A89="",B89=""),"",IF(B89="Activity",D89*(E89/100)*(1+N(F89)+N(G89)),D89*(E89/100)*H89))</f>
+        <f>IF(OR(A89="",B89=""),"",IF(B89="Activity",MAX(0,N(D89))*(MIN(100,MAX(0,N(E89)))/100)*(1+MAX(0,N(F89))+MAX(0,N(G89))),MAX(0,N(D89))*(MIN(100,MAX(0,N(E89)))/100)*H89))</f>
         <v/>
       </c>
     </row>
@@ -3970,7 +3987,7 @@
         <v/>
       </c>
       <c r="I90" s="22">
-        <f>IF(OR(A90="",B90=""),"",IF(B90="Activity",D90*(E90/100)*(1+N(F90)+N(G90)),D90*(E90/100)*H90))</f>
+        <f>IF(OR(A90="",B90=""),"",IF(B90="Activity",MAX(0,N(D90))*(MIN(100,MAX(0,N(E90)))/100)*(1+MAX(0,N(F90))+MAX(0,N(G90))),MAX(0,N(D90))*(MIN(100,MAX(0,N(E90)))/100)*H90))</f>
         <v/>
       </c>
     </row>
@@ -3987,7 +4004,7 @@
         <v/>
       </c>
       <c r="I91" s="22">
-        <f>IF(OR(A91="",B91=""),"",IF(B91="Activity",D91*(E91/100)*(1+N(F91)+N(G91)),D91*(E91/100)*H91))</f>
+        <f>IF(OR(A91="",B91=""),"",IF(B91="Activity",MAX(0,N(D91))*(MIN(100,MAX(0,N(E91)))/100)*(1+MAX(0,N(F91))+MAX(0,N(G91))),MAX(0,N(D91))*(MIN(100,MAX(0,N(E91)))/100)*H91))</f>
         <v/>
       </c>
     </row>
@@ -4004,7 +4021,7 @@
         <v/>
       </c>
       <c r="I92" s="22">
-        <f>IF(OR(A92="",B92=""),"",IF(B92="Activity",D92*(E92/100)*(1+N(F92)+N(G92)),D92*(E92/100)*H92))</f>
+        <f>IF(OR(A92="",B92=""),"",IF(B92="Activity",MAX(0,N(D92))*(MIN(100,MAX(0,N(E92)))/100)*(1+MAX(0,N(F92))+MAX(0,N(G92))),MAX(0,N(D92))*(MIN(100,MAX(0,N(E92)))/100)*H92))</f>
         <v/>
       </c>
     </row>
@@ -4021,7 +4038,7 @@
         <v/>
       </c>
       <c r="I93" s="22">
-        <f>IF(OR(A93="",B93=""),"",IF(B93="Activity",D93*(E93/100)*(1+N(F93)+N(G93)),D93*(E93/100)*H93))</f>
+        <f>IF(OR(A93="",B93=""),"",IF(B93="Activity",MAX(0,N(D93))*(MIN(100,MAX(0,N(E93)))/100)*(1+MAX(0,N(F93))+MAX(0,N(G93))),MAX(0,N(D93))*(MIN(100,MAX(0,N(E93)))/100)*H93))</f>
         <v/>
       </c>
     </row>
@@ -4038,7 +4055,7 @@
         <v/>
       </c>
       <c r="I94" s="22">
-        <f>IF(OR(A94="",B94=""),"",IF(B94="Activity",D94*(E94/100)*(1+N(F94)+N(G94)),D94*(E94/100)*H94))</f>
+        <f>IF(OR(A94="",B94=""),"",IF(B94="Activity",MAX(0,N(D94))*(MIN(100,MAX(0,N(E94)))/100)*(1+MAX(0,N(F94))+MAX(0,N(G94))),MAX(0,N(D94))*(MIN(100,MAX(0,N(E94)))/100)*H94))</f>
         <v/>
       </c>
     </row>
@@ -4055,7 +4072,7 @@
         <v/>
       </c>
       <c r="I95" s="22">
-        <f>IF(OR(A95="",B95=""),"",IF(B95="Activity",D95*(E95/100)*(1+N(F95)+N(G95)),D95*(E95/100)*H95))</f>
+        <f>IF(OR(A95="",B95=""),"",IF(B95="Activity",MAX(0,N(D95))*(MIN(100,MAX(0,N(E95)))/100)*(1+MAX(0,N(F95))+MAX(0,N(G95))),MAX(0,N(D95))*(MIN(100,MAX(0,N(E95)))/100)*H95))</f>
         <v/>
       </c>
     </row>
@@ -4072,7 +4089,7 @@
         <v/>
       </c>
       <c r="I96" s="22">
-        <f>IF(OR(A96="",B96=""),"",IF(B96="Activity",D96*(E96/100)*(1+N(F96)+N(G96)),D96*(E96/100)*H96))</f>
+        <f>IF(OR(A96="",B96=""),"",IF(B96="Activity",MAX(0,N(D96))*(MIN(100,MAX(0,N(E96)))/100)*(1+MAX(0,N(F96))+MAX(0,N(G96))),MAX(0,N(D96))*(MIN(100,MAX(0,N(E96)))/100)*H96))</f>
         <v/>
       </c>
     </row>
@@ -4089,7 +4106,7 @@
         <v/>
       </c>
       <c r="I97" s="22">
-        <f>IF(OR(A97="",B97=""),"",IF(B97="Activity",D97*(E97/100)*(1+N(F97)+N(G97)),D97*(E97/100)*H97))</f>
+        <f>IF(OR(A97="",B97=""),"",IF(B97="Activity",MAX(0,N(D97))*(MIN(100,MAX(0,N(E97)))/100)*(1+MAX(0,N(F97))+MAX(0,N(G97))),MAX(0,N(D97))*(MIN(100,MAX(0,N(E97)))/100)*H97))</f>
         <v/>
       </c>
     </row>
@@ -4106,7 +4123,7 @@
         <v/>
       </c>
       <c r="I98" s="22">
-        <f>IF(OR(A98="",B98=""),"",IF(B98="Activity",D98*(E98/100)*(1+N(F98)+N(G98)),D98*(E98/100)*H98))</f>
+        <f>IF(OR(A98="",B98=""),"",IF(B98="Activity",MAX(0,N(D98))*(MIN(100,MAX(0,N(E98)))/100)*(1+MAX(0,N(F98))+MAX(0,N(G98))),MAX(0,N(D98))*(MIN(100,MAX(0,N(E98)))/100)*H98))</f>
         <v/>
       </c>
     </row>
@@ -4123,7 +4140,7 @@
         <v/>
       </c>
       <c r="I99" s="22">
-        <f>IF(OR(A99="",B99=""),"",IF(B99="Activity",D99*(E99/100)*(1+N(F99)+N(G99)),D99*(E99/100)*H99))</f>
+        <f>IF(OR(A99="",B99=""),"",IF(B99="Activity",MAX(0,N(D99))*(MIN(100,MAX(0,N(E99)))/100)*(1+MAX(0,N(F99))+MAX(0,N(G99))),MAX(0,N(D99))*(MIN(100,MAX(0,N(E99)))/100)*H99))</f>
         <v/>
       </c>
     </row>
@@ -4140,7 +4157,7 @@
         <v/>
       </c>
       <c r="I100" s="22">
-        <f>IF(OR(A100="",B100=""),"",IF(B100="Activity",D100*(E100/100)*(1+N(F100)+N(G100)),D100*(E100/100)*H100))</f>
+        <f>IF(OR(A100="",B100=""),"",IF(B100="Activity",MAX(0,N(D100))*(MIN(100,MAX(0,N(E100)))/100)*(1+MAX(0,N(F100))+MAX(0,N(G100))),MAX(0,N(D100))*(MIN(100,MAX(0,N(E100)))/100)*H100))</f>
         <v/>
       </c>
     </row>
@@ -4157,7 +4174,7 @@
         <v/>
       </c>
       <c r="I101" s="22">
-        <f>IF(OR(A101="",B101=""),"",IF(B101="Activity",D101*(E101/100)*(1+N(F101)+N(G101)),D101*(E101/100)*H101))</f>
+        <f>IF(OR(A101="",B101=""),"",IF(B101="Activity",MAX(0,N(D101))*(MIN(100,MAX(0,N(E101)))/100)*(1+MAX(0,N(F101))+MAX(0,N(G101))),MAX(0,N(D101))*(MIN(100,MAX(0,N(E101)))/100)*H101))</f>
         <v/>
       </c>
     </row>
@@ -4174,7 +4191,7 @@
         <v/>
       </c>
       <c r="I102" s="22">
-        <f>IF(OR(A102="",B102=""),"",IF(B102="Activity",D102*(E102/100)*(1+N(F102)+N(G102)),D102*(E102/100)*H102))</f>
+        <f>IF(OR(A102="",B102=""),"",IF(B102="Activity",MAX(0,N(D102))*(MIN(100,MAX(0,N(E102)))/100)*(1+MAX(0,N(F102))+MAX(0,N(G102))),MAX(0,N(D102))*(MIN(100,MAX(0,N(E102)))/100)*H102))</f>
         <v/>
       </c>
     </row>
@@ -4191,7 +4208,7 @@
         <v/>
       </c>
       <c r="I103" s="22">
-        <f>IF(OR(A103="",B103=""),"",IF(B103="Activity",D103*(E103/100)*(1+N(F103)+N(G103)),D103*(E103/100)*H103))</f>
+        <f>IF(OR(A103="",B103=""),"",IF(B103="Activity",MAX(0,N(D103))*(MIN(100,MAX(0,N(E103)))/100)*(1+MAX(0,N(F103))+MAX(0,N(G103))),MAX(0,N(D103))*(MIN(100,MAX(0,N(E103)))/100)*H103))</f>
         <v/>
       </c>
     </row>
@@ -4208,7 +4225,7 @@
         <v/>
       </c>
       <c r="I104" s="22">
-        <f>IF(OR(A104="",B104=""),"",IF(B104="Activity",D104*(E104/100)*(1+N(F104)+N(G104)),D104*(E104/100)*H104))</f>
+        <f>IF(OR(A104="",B104=""),"",IF(B104="Activity",MAX(0,N(D104))*(MIN(100,MAX(0,N(E104)))/100)*(1+MAX(0,N(F104))+MAX(0,N(G104))),MAX(0,N(D104))*(MIN(100,MAX(0,N(E104)))/100)*H104))</f>
         <v/>
       </c>
     </row>
@@ -4225,7 +4242,7 @@
         <v/>
       </c>
       <c r="I105" s="22">
-        <f>IF(OR(A105="",B105=""),"",IF(B105="Activity",D105*(E105/100)*(1+N(F105)+N(G105)),D105*(E105/100)*H105))</f>
+        <f>IF(OR(A105="",B105=""),"",IF(B105="Activity",MAX(0,N(D105))*(MIN(100,MAX(0,N(E105)))/100)*(1+MAX(0,N(F105))+MAX(0,N(G105))),MAX(0,N(D105))*(MIN(100,MAX(0,N(E105)))/100)*H105))</f>
         <v/>
       </c>
     </row>
@@ -4242,7 +4259,7 @@
         <v/>
       </c>
       <c r="I106" s="22">
-        <f>IF(OR(A106="",B106=""),"",IF(B106="Activity",D106*(E106/100)*(1+N(F106)+N(G106)),D106*(E106/100)*H106))</f>
+        <f>IF(OR(A106="",B106=""),"",IF(B106="Activity",MAX(0,N(D106))*(MIN(100,MAX(0,N(E106)))/100)*(1+MAX(0,N(F106))+MAX(0,N(G106))),MAX(0,N(D106))*(MIN(100,MAX(0,N(E106)))/100)*H106))</f>
         <v/>
       </c>
     </row>
@@ -4259,7 +4276,7 @@
         <v/>
       </c>
       <c r="I107" s="22">
-        <f>IF(OR(A107="",B107=""),"",IF(B107="Activity",D107*(E107/100)*(1+N(F107)+N(G107)),D107*(E107/100)*H107))</f>
+        <f>IF(OR(A107="",B107=""),"",IF(B107="Activity",MAX(0,N(D107))*(MIN(100,MAX(0,N(E107)))/100)*(1+MAX(0,N(F107))+MAX(0,N(G107))),MAX(0,N(D107))*(MIN(100,MAX(0,N(E107)))/100)*H107))</f>
         <v/>
       </c>
     </row>
@@ -4276,7 +4293,7 @@
         <v/>
       </c>
       <c r="I108" s="22">
-        <f>IF(OR(A108="",B108=""),"",IF(B108="Activity",D108*(E108/100)*(1+N(F108)+N(G108)),D108*(E108/100)*H108))</f>
+        <f>IF(OR(A108="",B108=""),"",IF(B108="Activity",MAX(0,N(D108))*(MIN(100,MAX(0,N(E108)))/100)*(1+MAX(0,N(F108))+MAX(0,N(G108))),MAX(0,N(D108))*(MIN(100,MAX(0,N(E108)))/100)*H108))</f>
         <v/>
       </c>
     </row>
@@ -4293,7 +4310,7 @@
         <v/>
       </c>
       <c r="I109" s="22">
-        <f>IF(OR(A109="",B109=""),"",IF(B109="Activity",D109*(E109/100)*(1+N(F109)+N(G109)),D109*(E109/100)*H109))</f>
+        <f>IF(OR(A109="",B109=""),"",IF(B109="Activity",MAX(0,N(D109))*(MIN(100,MAX(0,N(E109)))/100)*(1+MAX(0,N(F109))+MAX(0,N(G109))),MAX(0,N(D109))*(MIN(100,MAX(0,N(E109)))/100)*H109))</f>
         <v/>
       </c>
     </row>
@@ -4310,7 +4327,7 @@
         <v/>
       </c>
       <c r="I110" s="22">
-        <f>IF(OR(A110="",B110=""),"",IF(B110="Activity",D110*(E110/100)*(1+N(F110)+N(G110)),D110*(E110/100)*H110))</f>
+        <f>IF(OR(A110="",B110=""),"",IF(B110="Activity",MAX(0,N(D110))*(MIN(100,MAX(0,N(E110)))/100)*(1+MAX(0,N(F110))+MAX(0,N(G110))),MAX(0,N(D110))*(MIN(100,MAX(0,N(E110)))/100)*H110))</f>
         <v/>
       </c>
     </row>
@@ -4327,7 +4344,7 @@
         <v/>
       </c>
       <c r="I111" s="22">
-        <f>IF(OR(A111="",B111=""),"",IF(B111="Activity",D111*(E111/100)*(1+N(F111)+N(G111)),D111*(E111/100)*H111))</f>
+        <f>IF(OR(A111="",B111=""),"",IF(B111="Activity",MAX(0,N(D111))*(MIN(100,MAX(0,N(E111)))/100)*(1+MAX(0,N(F111))+MAX(0,N(G111))),MAX(0,N(D111))*(MIN(100,MAX(0,N(E111)))/100)*H111))</f>
         <v/>
       </c>
     </row>
@@ -4344,7 +4361,7 @@
         <v/>
       </c>
       <c r="I112" s="22">
-        <f>IF(OR(A112="",B112=""),"",IF(B112="Activity",D112*(E112/100)*(1+N(F112)+N(G112)),D112*(E112/100)*H112))</f>
+        <f>IF(OR(A112="",B112=""),"",IF(B112="Activity",MAX(0,N(D112))*(MIN(100,MAX(0,N(E112)))/100)*(1+MAX(0,N(F112))+MAX(0,N(G112))),MAX(0,N(D112))*(MIN(100,MAX(0,N(E112)))/100)*H112))</f>
         <v/>
       </c>
     </row>
@@ -4361,7 +4378,7 @@
         <v/>
       </c>
       <c r="I113" s="22">
-        <f>IF(OR(A113="",B113=""),"",IF(B113="Activity",D113*(E113/100)*(1+N(F113)+N(G113)),D113*(E113/100)*H113))</f>
+        <f>IF(OR(A113="",B113=""),"",IF(B113="Activity",MAX(0,N(D113))*(MIN(100,MAX(0,N(E113)))/100)*(1+MAX(0,N(F113))+MAX(0,N(G113))),MAX(0,N(D113))*(MIN(100,MAX(0,N(E113)))/100)*H113))</f>
         <v/>
       </c>
     </row>
@@ -4378,7 +4395,7 @@
         <v/>
       </c>
       <c r="I114" s="22">
-        <f>IF(OR(A114="",B114=""),"",IF(B114="Activity",D114*(E114/100)*(1+N(F114)+N(G114)),D114*(E114/100)*H114))</f>
+        <f>IF(OR(A114="",B114=""),"",IF(B114="Activity",MAX(0,N(D114))*(MIN(100,MAX(0,N(E114)))/100)*(1+MAX(0,N(F114))+MAX(0,N(G114))),MAX(0,N(D114))*(MIN(100,MAX(0,N(E114)))/100)*H114))</f>
         <v/>
       </c>
     </row>
@@ -4395,7 +4412,7 @@
         <v/>
       </c>
       <c r="I115" s="22">
-        <f>IF(OR(A115="",B115=""),"",IF(B115="Activity",D115*(E115/100)*(1+N(F115)+N(G115)),D115*(E115/100)*H115))</f>
+        <f>IF(OR(A115="",B115=""),"",IF(B115="Activity",MAX(0,N(D115))*(MIN(100,MAX(0,N(E115)))/100)*(1+MAX(0,N(F115))+MAX(0,N(G115))),MAX(0,N(D115))*(MIN(100,MAX(0,N(E115)))/100)*H115))</f>
         <v/>
       </c>
     </row>
@@ -4412,7 +4429,7 @@
         <v/>
       </c>
       <c r="I116" s="22">
-        <f>IF(OR(A116="",B116=""),"",IF(B116="Activity",D116*(E116/100)*(1+N(F116)+N(G116)),D116*(E116/100)*H116))</f>
+        <f>IF(OR(A116="",B116=""),"",IF(B116="Activity",MAX(0,N(D116))*(MIN(100,MAX(0,N(E116)))/100)*(1+MAX(0,N(F116))+MAX(0,N(G116))),MAX(0,N(D116))*(MIN(100,MAX(0,N(E116)))/100)*H116))</f>
         <v/>
       </c>
     </row>
@@ -4429,7 +4446,7 @@
         <v/>
       </c>
       <c r="I117" s="22">
-        <f>IF(OR(A117="",B117=""),"",IF(B117="Activity",D117*(E117/100)*(1+N(F117)+N(G117)),D117*(E117/100)*H117))</f>
+        <f>IF(OR(A117="",B117=""),"",IF(B117="Activity",MAX(0,N(D117))*(MIN(100,MAX(0,N(E117)))/100)*(1+MAX(0,N(F117))+MAX(0,N(G117))),MAX(0,N(D117))*(MIN(100,MAX(0,N(E117)))/100)*H117))</f>
         <v/>
       </c>
     </row>
@@ -4446,7 +4463,7 @@
         <v/>
       </c>
       <c r="I118" s="22">
-        <f>IF(OR(A118="",B118=""),"",IF(B118="Activity",D118*(E118/100)*(1+N(F118)+N(G118)),D118*(E118/100)*H118))</f>
+        <f>IF(OR(A118="",B118=""),"",IF(B118="Activity",MAX(0,N(D118))*(MIN(100,MAX(0,N(E118)))/100)*(1+MAX(0,N(F118))+MAX(0,N(G118))),MAX(0,N(D118))*(MIN(100,MAX(0,N(E118)))/100)*H118))</f>
         <v/>
       </c>
     </row>
@@ -4463,7 +4480,7 @@
         <v/>
       </c>
       <c r="I119" s="22">
-        <f>IF(OR(A119="",B119=""),"",IF(B119="Activity",D119*(E119/100)*(1+N(F119)+N(G119)),D119*(E119/100)*H119))</f>
+        <f>IF(OR(A119="",B119=""),"",IF(B119="Activity",MAX(0,N(D119))*(MIN(100,MAX(0,N(E119)))/100)*(1+MAX(0,N(F119))+MAX(0,N(G119))),MAX(0,N(D119))*(MIN(100,MAX(0,N(E119)))/100)*H119))</f>
         <v/>
       </c>
     </row>
@@ -4480,7 +4497,7 @@
         <v/>
       </c>
       <c r="I120" s="22">
-        <f>IF(OR(A120="",B120=""),"",IF(B120="Activity",D120*(E120/100)*(1+N(F120)+N(G120)),D120*(E120/100)*H120))</f>
+        <f>IF(OR(A120="",B120=""),"",IF(B120="Activity",MAX(0,N(D120))*(MIN(100,MAX(0,N(E120)))/100)*(1+MAX(0,N(F120))+MAX(0,N(G120))),MAX(0,N(D120))*(MIN(100,MAX(0,N(E120)))/100)*H120))</f>
         <v/>
       </c>
     </row>
@@ -4497,7 +4514,7 @@
         <v/>
       </c>
       <c r="I121" s="22">
-        <f>IF(OR(A121="",B121=""),"",IF(B121="Activity",D121*(E121/100)*(1+N(F121)+N(G121)),D121*(E121/100)*H121))</f>
+        <f>IF(OR(A121="",B121=""),"",IF(B121="Activity",MAX(0,N(D121))*(MIN(100,MAX(0,N(E121)))/100)*(1+MAX(0,N(F121))+MAX(0,N(G121))),MAX(0,N(D121))*(MIN(100,MAX(0,N(E121)))/100)*H121))</f>
         <v/>
       </c>
     </row>
@@ -4514,7 +4531,7 @@
         <v/>
       </c>
       <c r="I122" s="22">
-        <f>IF(OR(A122="",B122=""),"",IF(B122="Activity",D122*(E122/100)*(1+N(F122)+N(G122)),D122*(E122/100)*H122))</f>
+        <f>IF(OR(A122="",B122=""),"",IF(B122="Activity",MAX(0,N(D122))*(MIN(100,MAX(0,N(E122)))/100)*(1+MAX(0,N(F122))+MAX(0,N(G122))),MAX(0,N(D122))*(MIN(100,MAX(0,N(E122)))/100)*H122))</f>
         <v/>
       </c>
     </row>
@@ -4531,7 +4548,7 @@
         <v/>
       </c>
       <c r="I123" s="22">
-        <f>IF(OR(A123="",B123=""),"",IF(B123="Activity",D123*(E123/100)*(1+N(F123)+N(G123)),D123*(E123/100)*H123))</f>
+        <f>IF(OR(A123="",B123=""),"",IF(B123="Activity",MAX(0,N(D123))*(MIN(100,MAX(0,N(E123)))/100)*(1+MAX(0,N(F123))+MAX(0,N(G123))),MAX(0,N(D123))*(MIN(100,MAX(0,N(E123)))/100)*H123))</f>
         <v/>
       </c>
     </row>
@@ -4548,7 +4565,7 @@
         <v/>
       </c>
       <c r="I124" s="22">
-        <f>IF(OR(A124="",B124=""),"",IF(B124="Activity",D124*(E124/100)*(1+N(F124)+N(G124)),D124*(E124/100)*H124))</f>
+        <f>IF(OR(A124="",B124=""),"",IF(B124="Activity",MAX(0,N(D124))*(MIN(100,MAX(0,N(E124)))/100)*(1+MAX(0,N(F124))+MAX(0,N(G124))),MAX(0,N(D124))*(MIN(100,MAX(0,N(E124)))/100)*H124))</f>
         <v/>
       </c>
     </row>
@@ -4565,7 +4582,7 @@
         <v/>
       </c>
       <c r="I125" s="22">
-        <f>IF(OR(A125="",B125=""),"",IF(B125="Activity",D125*(E125/100)*(1+N(F125)+N(G125)),D125*(E125/100)*H125))</f>
+        <f>IF(OR(A125="",B125=""),"",IF(B125="Activity",MAX(0,N(D125))*(MIN(100,MAX(0,N(E125)))/100)*(1+MAX(0,N(F125))+MAX(0,N(G125))),MAX(0,N(D125))*(MIN(100,MAX(0,N(E125)))/100)*H125))</f>
         <v/>
       </c>
     </row>
@@ -4582,7 +4599,7 @@
         <v/>
       </c>
       <c r="I126" s="22">
-        <f>IF(OR(A126="",B126=""),"",IF(B126="Activity",D126*(E126/100)*(1+N(F126)+N(G126)),D126*(E126/100)*H126))</f>
+        <f>IF(OR(A126="",B126=""),"",IF(B126="Activity",MAX(0,N(D126))*(MIN(100,MAX(0,N(E126)))/100)*(1+MAX(0,N(F126))+MAX(0,N(G126))),MAX(0,N(D126))*(MIN(100,MAX(0,N(E126)))/100)*H126))</f>
         <v/>
       </c>
     </row>
@@ -4599,7 +4616,7 @@
         <v/>
       </c>
       <c r="I127" s="22">
-        <f>IF(OR(A127="",B127=""),"",IF(B127="Activity",D127*(E127/100)*(1+N(F127)+N(G127)),D127*(E127/100)*H127))</f>
+        <f>IF(OR(A127="",B127=""),"",IF(B127="Activity",MAX(0,N(D127))*(MIN(100,MAX(0,N(E127)))/100)*(1+MAX(0,N(F127))+MAX(0,N(G127))),MAX(0,N(D127))*(MIN(100,MAX(0,N(E127)))/100)*H127))</f>
         <v/>
       </c>
     </row>
@@ -4616,7 +4633,7 @@
         <v/>
       </c>
       <c r="I128" s="22">
-        <f>IF(OR(A128="",B128=""),"",IF(B128="Activity",D128*(E128/100)*(1+N(F128)+N(G128)),D128*(E128/100)*H128))</f>
+        <f>IF(OR(A128="",B128=""),"",IF(B128="Activity",MAX(0,N(D128))*(MIN(100,MAX(0,N(E128)))/100)*(1+MAX(0,N(F128))+MAX(0,N(G128))),MAX(0,N(D128))*(MIN(100,MAX(0,N(E128)))/100)*H128))</f>
         <v/>
       </c>
     </row>
@@ -4633,7 +4650,7 @@
         <v/>
       </c>
       <c r="I129" s="22">
-        <f>IF(OR(A129="",B129=""),"",IF(B129="Activity",D129*(E129/100)*(1+N(F129)+N(G129)),D129*(E129/100)*H129))</f>
+        <f>IF(OR(A129="",B129=""),"",IF(B129="Activity",MAX(0,N(D129))*(MIN(100,MAX(0,N(E129)))/100)*(1+MAX(0,N(F129))+MAX(0,N(G129))),MAX(0,N(D129))*(MIN(100,MAX(0,N(E129)))/100)*H129))</f>
         <v/>
       </c>
     </row>
@@ -4650,7 +4667,7 @@
         <v/>
       </c>
       <c r="I130" s="22">
-        <f>IF(OR(A130="",B130=""),"",IF(B130="Activity",D130*(E130/100)*(1+N(F130)+N(G130)),D130*(E130/100)*H130))</f>
+        <f>IF(OR(A130="",B130=""),"",IF(B130="Activity",MAX(0,N(D130))*(MIN(100,MAX(0,N(E130)))/100)*(1+MAX(0,N(F130))+MAX(0,N(G130))),MAX(0,N(D130))*(MIN(100,MAX(0,N(E130)))/100)*H130))</f>
         <v/>
       </c>
     </row>
@@ -4667,7 +4684,7 @@
         <v/>
       </c>
       <c r="I131" s="22">
-        <f>IF(OR(A131="",B131=""),"",IF(B131="Activity",D131*(E131/100)*(1+N(F131)+N(G131)),D131*(E131/100)*H131))</f>
+        <f>IF(OR(A131="",B131=""),"",IF(B131="Activity",MAX(0,N(D131))*(MIN(100,MAX(0,N(E131)))/100)*(1+MAX(0,N(F131))+MAX(0,N(G131))),MAX(0,N(D131))*(MIN(100,MAX(0,N(E131)))/100)*H131))</f>
         <v/>
       </c>
     </row>
@@ -4684,7 +4701,7 @@
         <v/>
       </c>
       <c r="I132" s="22">
-        <f>IF(OR(A132="",B132=""),"",IF(B132="Activity",D132*(E132/100)*(1+N(F132)+N(G132)),D132*(E132/100)*H132))</f>
+        <f>IF(OR(A132="",B132=""),"",IF(B132="Activity",MAX(0,N(D132))*(MIN(100,MAX(0,N(E132)))/100)*(1+MAX(0,N(F132))+MAX(0,N(G132))),MAX(0,N(D132))*(MIN(100,MAX(0,N(E132)))/100)*H132))</f>
         <v/>
       </c>
     </row>
@@ -4701,7 +4718,7 @@
         <v/>
       </c>
       <c r="I133" s="22">
-        <f>IF(OR(A133="",B133=""),"",IF(B133="Activity",D133*(E133/100)*(1+N(F133)+N(G133)),D133*(E133/100)*H133))</f>
+        <f>IF(OR(A133="",B133=""),"",IF(B133="Activity",MAX(0,N(D133))*(MIN(100,MAX(0,N(E133)))/100)*(1+MAX(0,N(F133))+MAX(0,N(G133))),MAX(0,N(D133))*(MIN(100,MAX(0,N(E133)))/100)*H133))</f>
         <v/>
       </c>
     </row>
@@ -4718,7 +4735,7 @@
         <v/>
       </c>
       <c r="I134" s="22">
-        <f>IF(OR(A134="",B134=""),"",IF(B134="Activity",D134*(E134/100)*(1+N(F134)+N(G134)),D134*(E134/100)*H134))</f>
+        <f>IF(OR(A134="",B134=""),"",IF(B134="Activity",MAX(0,N(D134))*(MIN(100,MAX(0,N(E134)))/100)*(1+MAX(0,N(F134))+MAX(0,N(G134))),MAX(0,N(D134))*(MIN(100,MAX(0,N(E134)))/100)*H134))</f>
         <v/>
       </c>
     </row>
@@ -4735,7 +4752,7 @@
         <v/>
       </c>
       <c r="I135" s="22">
-        <f>IF(OR(A135="",B135=""),"",IF(B135="Activity",D135*(E135/100)*(1+N(F135)+N(G135)),D135*(E135/100)*H135))</f>
+        <f>IF(OR(A135="",B135=""),"",IF(B135="Activity",MAX(0,N(D135))*(MIN(100,MAX(0,N(E135)))/100)*(1+MAX(0,N(F135))+MAX(0,N(G135))),MAX(0,N(D135))*(MIN(100,MAX(0,N(E135)))/100)*H135))</f>
         <v/>
       </c>
     </row>
@@ -4752,7 +4769,7 @@
         <v/>
       </c>
       <c r="I136" s="22">
-        <f>IF(OR(A136="",B136=""),"",IF(B136="Activity",D136*(E136/100)*(1+N(F136)+N(G136)),D136*(E136/100)*H136))</f>
+        <f>IF(OR(A136="",B136=""),"",IF(B136="Activity",MAX(0,N(D136))*(MIN(100,MAX(0,N(E136)))/100)*(1+MAX(0,N(F136))+MAX(0,N(G136))),MAX(0,N(D136))*(MIN(100,MAX(0,N(E136)))/100)*H136))</f>
         <v/>
       </c>
     </row>
@@ -4769,7 +4786,7 @@
         <v/>
       </c>
       <c r="I137" s="22">
-        <f>IF(OR(A137="",B137=""),"",IF(B137="Activity",D137*(E137/100)*(1+N(F137)+N(G137)),D137*(E137/100)*H137))</f>
+        <f>IF(OR(A137="",B137=""),"",IF(B137="Activity",MAX(0,N(D137))*(MIN(100,MAX(0,N(E137)))/100)*(1+MAX(0,N(F137))+MAX(0,N(G137))),MAX(0,N(D137))*(MIN(100,MAX(0,N(E137)))/100)*H137))</f>
         <v/>
       </c>
     </row>
@@ -4786,7 +4803,7 @@
         <v/>
       </c>
       <c r="I138" s="22">
-        <f>IF(OR(A138="",B138=""),"",IF(B138="Activity",D138*(E138/100)*(1+N(F138)+N(G138)),D138*(E138/100)*H138))</f>
+        <f>IF(OR(A138="",B138=""),"",IF(B138="Activity",MAX(0,N(D138))*(MIN(100,MAX(0,N(E138)))/100)*(1+MAX(0,N(F138))+MAX(0,N(G138))),MAX(0,N(D138))*(MIN(100,MAX(0,N(E138)))/100)*H138))</f>
         <v/>
       </c>
     </row>
@@ -4803,7 +4820,7 @@
         <v/>
       </c>
       <c r="I139" s="22">
-        <f>IF(OR(A139="",B139=""),"",IF(B139="Activity",D139*(E139/100)*(1+N(F139)+N(G139)),D139*(E139/100)*H139))</f>
+        <f>IF(OR(A139="",B139=""),"",IF(B139="Activity",MAX(0,N(D139))*(MIN(100,MAX(0,N(E139)))/100)*(1+MAX(0,N(F139))+MAX(0,N(G139))),MAX(0,N(D139))*(MIN(100,MAX(0,N(E139)))/100)*H139))</f>
         <v/>
       </c>
     </row>
@@ -4820,7 +4837,7 @@
         <v/>
       </c>
       <c r="I140" s="22">
-        <f>IF(OR(A140="",B140=""),"",IF(B140="Activity",D140*(E140/100)*(1+N(F140)+N(G140)),D140*(E140/100)*H140))</f>
+        <f>IF(OR(A140="",B140=""),"",IF(B140="Activity",MAX(0,N(D140))*(MIN(100,MAX(0,N(E140)))/100)*(1+MAX(0,N(F140))+MAX(0,N(G140))),MAX(0,N(D140))*(MIN(100,MAX(0,N(E140)))/100)*H140))</f>
         <v/>
       </c>
     </row>
@@ -4837,7 +4854,7 @@
         <v/>
       </c>
       <c r="I141" s="22">
-        <f>IF(OR(A141="",B141=""),"",IF(B141="Activity",D141*(E141/100)*(1+N(F141)+N(G141)),D141*(E141/100)*H141))</f>
+        <f>IF(OR(A141="",B141=""),"",IF(B141="Activity",MAX(0,N(D141))*(MIN(100,MAX(0,N(E141)))/100)*(1+MAX(0,N(F141))+MAX(0,N(G141))),MAX(0,N(D141))*(MIN(100,MAX(0,N(E141)))/100)*H141))</f>
         <v/>
       </c>
     </row>
@@ -4854,7 +4871,7 @@
         <v/>
       </c>
       <c r="I142" s="22">
-        <f>IF(OR(A142="",B142=""),"",IF(B142="Activity",D142*(E142/100)*(1+N(F142)+N(G142)),D142*(E142/100)*H142))</f>
+        <f>IF(OR(A142="",B142=""),"",IF(B142="Activity",MAX(0,N(D142))*(MIN(100,MAX(0,N(E142)))/100)*(1+MAX(0,N(F142))+MAX(0,N(G142))),MAX(0,N(D142))*(MIN(100,MAX(0,N(E142)))/100)*H142))</f>
         <v/>
       </c>
     </row>
@@ -4871,7 +4888,7 @@
         <v/>
       </c>
       <c r="I143" s="22">
-        <f>IF(OR(A143="",B143=""),"",IF(B143="Activity",D143*(E143/100)*(1+N(F143)+N(G143)),D143*(E143/100)*H143))</f>
+        <f>IF(OR(A143="",B143=""),"",IF(B143="Activity",MAX(0,N(D143))*(MIN(100,MAX(0,N(E143)))/100)*(1+MAX(0,N(F143))+MAX(0,N(G143))),MAX(0,N(D143))*(MIN(100,MAX(0,N(E143)))/100)*H143))</f>
         <v/>
       </c>
     </row>
@@ -4888,7 +4905,7 @@
         <v/>
       </c>
       <c r="I144" s="22">
-        <f>IF(OR(A144="",B144=""),"",IF(B144="Activity",D144*(E144/100)*(1+N(F144)+N(G144)),D144*(E144/100)*H144))</f>
+        <f>IF(OR(A144="",B144=""),"",IF(B144="Activity",MAX(0,N(D144))*(MIN(100,MAX(0,N(E144)))/100)*(1+MAX(0,N(F144))+MAX(0,N(G144))),MAX(0,N(D144))*(MIN(100,MAX(0,N(E144)))/100)*H144))</f>
         <v/>
       </c>
     </row>
@@ -4905,7 +4922,7 @@
         <v/>
       </c>
       <c r="I145" s="22">
-        <f>IF(OR(A145="",B145=""),"",IF(B145="Activity",D145*(E145/100)*(1+N(F145)+N(G145)),D145*(E145/100)*H145))</f>
+        <f>IF(OR(A145="",B145=""),"",IF(B145="Activity",MAX(0,N(D145))*(MIN(100,MAX(0,N(E145)))/100)*(1+MAX(0,N(F145))+MAX(0,N(G145))),MAX(0,N(D145))*(MIN(100,MAX(0,N(E145)))/100)*H145))</f>
         <v/>
       </c>
     </row>
@@ -4922,7 +4939,7 @@
         <v/>
       </c>
       <c r="I146" s="22">
-        <f>IF(OR(A146="",B146=""),"",IF(B146="Activity",D146*(E146/100)*(1+N(F146)+N(G146)),D146*(E146/100)*H146))</f>
+        <f>IF(OR(A146="",B146=""),"",IF(B146="Activity",MAX(0,N(D146))*(MIN(100,MAX(0,N(E146)))/100)*(1+MAX(0,N(F146))+MAX(0,N(G146))),MAX(0,N(D146))*(MIN(100,MAX(0,N(E146)))/100)*H146))</f>
         <v/>
       </c>
     </row>
@@ -4939,7 +4956,7 @@
         <v/>
       </c>
       <c r="I147" s="22">
-        <f>IF(OR(A147="",B147=""),"",IF(B147="Activity",D147*(E147/100)*(1+N(F147)+N(G147)),D147*(E147/100)*H147))</f>
+        <f>IF(OR(A147="",B147=""),"",IF(B147="Activity",MAX(0,N(D147))*(MIN(100,MAX(0,N(E147)))/100)*(1+MAX(0,N(F147))+MAX(0,N(G147))),MAX(0,N(D147))*(MIN(100,MAX(0,N(E147)))/100)*H147))</f>
         <v/>
       </c>
     </row>
@@ -4956,7 +4973,7 @@
         <v/>
       </c>
       <c r="I148" s="22">
-        <f>IF(OR(A148="",B148=""),"",IF(B148="Activity",D148*(E148/100)*(1+N(F148)+N(G148)),D148*(E148/100)*H148))</f>
+        <f>IF(OR(A148="",B148=""),"",IF(B148="Activity",MAX(0,N(D148))*(MIN(100,MAX(0,N(E148)))/100)*(1+MAX(0,N(F148))+MAX(0,N(G148))),MAX(0,N(D148))*(MIN(100,MAX(0,N(E148)))/100)*H148))</f>
         <v/>
       </c>
     </row>
@@ -4973,7 +4990,7 @@
         <v/>
       </c>
       <c r="I149" s="22">
-        <f>IF(OR(A149="",B149=""),"",IF(B149="Activity",D149*(E149/100)*(1+N(F149)+N(G149)),D149*(E149/100)*H149))</f>
+        <f>IF(OR(A149="",B149=""),"",IF(B149="Activity",MAX(0,N(D149))*(MIN(100,MAX(0,N(E149)))/100)*(1+MAX(0,N(F149))+MAX(0,N(G149))),MAX(0,N(D149))*(MIN(100,MAX(0,N(E149)))/100)*H149))</f>
         <v/>
       </c>
     </row>
@@ -4990,7 +5007,7 @@
         <v/>
       </c>
       <c r="I150" s="22">
-        <f>IF(OR(A150="",B150=""),"",IF(B150="Activity",D150*(E150/100)*(1+N(F150)+N(G150)),D150*(E150/100)*H150))</f>
+        <f>IF(OR(A150="",B150=""),"",IF(B150="Activity",MAX(0,N(D150))*(MIN(100,MAX(0,N(E150)))/100)*(1+MAX(0,N(F150))+MAX(0,N(G150))),MAX(0,N(D150))*(MIN(100,MAX(0,N(E150)))/100)*H150))</f>
         <v/>
       </c>
     </row>
@@ -5007,7 +5024,7 @@
         <v/>
       </c>
       <c r="I151" s="22">
-        <f>IF(OR(A151="",B151=""),"",IF(B151="Activity",D151*(E151/100)*(1+N(F151)+N(G151)),D151*(E151/100)*H151))</f>
+        <f>IF(OR(A151="",B151=""),"",IF(B151="Activity",MAX(0,N(D151))*(MIN(100,MAX(0,N(E151)))/100)*(1+MAX(0,N(F151))+MAX(0,N(G151))),MAX(0,N(D151))*(MIN(100,MAX(0,N(E151)))/100)*H151))</f>
         <v/>
       </c>
     </row>

</xml_diff>